<commit_message>
Add every individual CAA/WME/UTA agent (Feb-Mar 2026 outreach)
Searched sent mail to agency domains and extracted all ~66 named agents
Norman cold-emailed across CAA, WME (agency + Entertainment), and UTA in
Feb-Mar 2026 (the 'NCAA Acquisition + Production' blast) - mostly one-way
sends with no reply. Replaces the earlier firm-level rollup with a
dedicated Agency Outreach category, each agent flagged responded vs.
no-reply for follow-up. Includes Ari Emanuel (WME CEO), Bryan Lourd,
Rick Kurtzman, and the responded set (Hess, Laur, Lucas, Nettler,
Sherman, Jasper, Volchok, Tim Curtis, etc.).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ajJRqKa1DUy4iKHJKPEi3
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-08-12-cinderella-contacts.xlsx
+++ b/cinderella/Outputs/2026-08-12-cinderella-contacts.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G185"/>
+  <dimension ref="A1:G253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6519,7 +6519,7 @@
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>CAA</t>
+          <t>CAA / WME / UTA individual agents</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
@@ -6529,160 +6529,160 @@
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>Bryan Lourd, Rick Kurtzman, Ethan Kurtzman, C. Carino, J. Darmody, J. MacGregor, T. Brennan</t>
+          <t>~75 named agents — see dedicated 'Agency Outreach' category below</t>
         </is>
       </c>
       <c r="D172" s="3" t="inlineStr">
         <is>
-          <t>blourd@caa.com</t>
+          <t>(various)</t>
         </is>
       </c>
       <c r="E172" s="3" t="inlineStr">
         <is>
-          <t>Feb 15+ agency blast</t>
+          <t>Feb–Mar 2026 blast</t>
         </is>
       </c>
       <c r="F172" s="3" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="G172" s="3" t="inlineStr">
         <is>
-          <t>Mostly no response — a few opens</t>
+          <t>See Agency Outreach category</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>WME Entertainment</t>
+          <t>Range Media Partners</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>Agency</t>
+          <t>Mgmt/agency</t>
         </is>
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>B. Slater, T. Curtis, D. Greenberg, H. Reisch, J. Lesh, N. Towne, S. Mark, W. Lowery, +</t>
+          <t>Kevin Hussey (Casey Affleck's mgr), Dave Bugliari, P. Orr, A. Glasgow, R. Astphan</t>
         </is>
       </c>
       <c r="D173" s="3" t="inlineStr">
         <is>
-          <t>bslater@wmeentertainment.com</t>
+          <t>khussey@rangemp.com</t>
         </is>
       </c>
       <c r="E173" s="3" t="inlineStr">
         <is>
-          <t>Feb 14-16 blast</t>
+          <t>Feb 14 blast</t>
         </is>
       </c>
       <c r="F173" s="3" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="G173" s="3" t="inlineStr">
         <is>
-          <t>No response</t>
+          <t>RESPONDED (Hussey/Glasgow) — revisit</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>WME (agency)</t>
+          <t>Octagon</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>Agency</t>
+          <t>Sports agency</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>M. Jasper (+assistant), M. Berkowitz, S. Rabinowitz</t>
+          <t>Jeff Austin</t>
         </is>
       </c>
       <c r="D174" s="3" t="inlineStr">
         <is>
-          <t>mberkowitz@wmeagency.com</t>
+          <t>jeff.austin@octagon.com</t>
         </is>
       </c>
       <c r="E174" s="3" t="inlineStr">
         <is>
-          <t>Feb-Mar blast</t>
+          <t>Feb 16 blast</t>
         </is>
       </c>
       <c r="F174" s="3" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="G174" s="3" t="inlineStr">
         <is>
-          <t>M. Jasper RESPONDED</t>
+          <t>No response</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>United Talent (UTA)</t>
+          <t>Untitled Entertainment</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>Agency</t>
+          <t>Mgmt</t>
         </is>
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>K. Volchok, J. Barber, N. Gates, B. Lazarus, D. Duchon, K. Lubeck, J. Lawson, S. Sacks, +</t>
+          <t>P. Murray</t>
         </is>
       </c>
       <c r="D175" s="3" t="inlineStr">
         <is>
-          <t>volchokk@unitedtalent.com</t>
+          <t>pmurray@untitledent.com</t>
         </is>
       </c>
       <c r="E175" s="3" t="inlineStr">
         <is>
-          <t>Feb 14-16 blast</t>
+          <t>Feb 15 blast</t>
         </is>
       </c>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="G175" s="3" t="inlineStr">
         <is>
-          <t>K. Volchok RESPONDED</t>
+          <t>RESPONDED</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>Range Media Partners</t>
+          <t>Independent Artists Media</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>Mgmt/agency</t>
+          <t>Mgmt</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
-          <t>Kevin Hussey (Casey Affleck's mgr), Dave Bugliari, P. Orr, A. Glasgow, R. Astphan</t>
+          <t>Dave, Alex</t>
         </is>
       </c>
       <c r="D176" s="3" t="inlineStr">
         <is>
-          <t>khussey@rangemp.com</t>
+          <t>dave@independentartistsmedia.com</t>
         </is>
       </c>
       <c r="E176" s="3" t="inlineStr">
@@ -6697,39 +6697,39 @@
       </c>
       <c r="G176" s="3" t="inlineStr">
         <is>
-          <t>RESPONDED (Hussey/Glasgow) — revisit</t>
+          <t>RESPONDED</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>Octagon</t>
+          <t>Red Light Management</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>Sports agency</t>
+          <t>Music mgmt</t>
         </is>
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>Jeff Austin</t>
+          <t>Coran Capshaw</t>
         </is>
       </c>
       <c r="D177" s="3" t="inlineStr">
         <is>
-          <t>jeff.austin@octagon.com</t>
+          <t>coran.capshaw@redlightmanagement.com</t>
         </is>
       </c>
       <c r="E177" s="3" t="inlineStr">
         <is>
-          <t>Feb 16 blast</t>
+          <t>Feb 15 blast</t>
         </is>
       </c>
       <c r="F177" s="3" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="G177" s="3" t="inlineStr">
@@ -6741,32 +6741,32 @@
     <row r="178">
       <c r="A178" s="3" t="inlineStr">
         <is>
-          <t>Untitled Entertainment</t>
+          <t>EB Media PR</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>Mgmt</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>P. Murray</t>
+          <t>Joseph, Ebie</t>
         </is>
       </c>
       <c r="D178" s="3" t="inlineStr">
         <is>
-          <t>pmurray@untitledent.com</t>
+          <t>ebie@ebmediapr.com</t>
         </is>
       </c>
       <c r="E178" s="3" t="inlineStr">
         <is>
-          <t>Feb 15 blast</t>
+          <t>Feb 16 blast</t>
         </is>
       </c>
       <c r="F178" s="3" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="G178" s="3" t="inlineStr">
@@ -6778,271 +6778,2758 @@
     <row r="179">
       <c r="A179" s="3" t="inlineStr">
         <is>
-          <t>Independent Artists Media</t>
+          <t>Other mgmt/PR (Feb blast)</t>
         </is>
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>Mgmt</t>
+          <t>Mgmt/PR</t>
         </is>
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>Dave, Alex</t>
+          <t>Kipperman, The AMG, Montag Group, Neal Agency, TCC, KP Ent, Make Wake, Yumkas, CSC Biz Mgmt, Price Mgmt, Rowe PR, Rogers&amp;Cowan (Nierob), Leverage, Media4Mgmt, LB Ent</t>
         </is>
       </c>
       <c r="D179" s="3" t="inlineStr">
         <is>
-          <t>dave@independentartistsmedia.com</t>
+          <t>(various)</t>
         </is>
       </c>
       <c r="E179" s="3" t="inlineStr">
         <is>
-          <t>Feb 14 blast</t>
+          <t>Feb 15 blast — see raw list</t>
         </is>
       </c>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="G179" s="3" t="inlineStr">
         <is>
-          <t>RESPONDED</t>
+          <t>Mostly no response</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="3" t="inlineStr">
         <is>
-          <t>Red Light Management</t>
+          <t>Andrew Schulz (camp)</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>Music mgmt</t>
+          <t>Comedian/talent</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>Coran Capshaw</t>
+          <t>Andrew, Dov, Tanya</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
         <is>
-          <t>coran.capshaw@redlightmanagement.com</t>
+          <t>andrew@theandrewschulz.com</t>
         </is>
       </c>
       <c r="E180" s="3" t="inlineStr">
         <is>
-          <t>Feb 15 blast</t>
+          <t>Cold outreach</t>
         </is>
       </c>
       <c r="F180" s="3" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="G180" s="3" t="inlineStr">
         <is>
-          <t>No response</t>
+          <t>Cold — comedian target</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="3" t="inlineStr">
         <is>
-          <t>EB Media PR</t>
+          <t>Schools — additional cold</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>College AD/coach</t>
         </is>
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>Joseph, Ebie</t>
+          <t>Holy Cross (Johnson/Paulsen/Rawlings), Stonehill (Kraus), UMBC (Lawson), Loyola (Blue), Coll. of Charleston (Harriman), Northeastern (Janning), BU (Quinn), UPenn</t>
         </is>
       </c>
       <c r="D181" s="3" t="inlineStr">
         <is>
-          <t>ebie@ebmediapr.com</t>
+          <t>(various .edu)</t>
         </is>
       </c>
       <c r="E181" s="3" t="inlineStr">
         <is>
-          <t>Feb 16 blast</t>
+          <t>Feb–Aug outreach</t>
         </is>
       </c>
       <c r="F181" s="3" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="G181" s="3" t="inlineStr">
         <is>
-          <t>RESPONDED</t>
+          <t>Mixed — BU responded; rest cold</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="3" t="inlineStr">
         <is>
-          <t>Other mgmt/PR (Feb blast)</t>
+          <t>O'Melveny &amp; Myers</t>
         </is>
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>Mgmt/PR</t>
+          <t>Law firm</t>
         </is>
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>Kipperman, The AMG, Montag Group, Neal Agency, TCC, KP Ent, Make Wake, Yumkas, CSC Biz Mgmt, Price Mgmt, Rowe PR, Rogers&amp;Cowan (Nierob), Leverage, Media4Mgmt, LB Ent</t>
+          <t>Aronson, Reinstein, Afner</t>
         </is>
       </c>
       <c r="D182" s="3" t="inlineStr">
         <is>
-          <t>(various)</t>
+          <t>baronson@omm.com</t>
         </is>
       </c>
       <c r="E182" s="3" t="inlineStr">
         <is>
-          <t>Feb 15 blast — see raw list</t>
+          <t>Cold outreach</t>
         </is>
       </c>
       <c r="F182" s="3" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="G182" s="3" t="inlineStr">
         <is>
-          <t>Mostly no response</t>
+          <t>Cold</t>
         </is>
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="3" t="inlineStr">
-        <is>
-          <t>Andrew Schulz (camp)</t>
-        </is>
-      </c>
-      <c r="B183" s="3" t="inlineStr">
-        <is>
-          <t>Comedian/talent</t>
-        </is>
-      </c>
-      <c r="C183" s="3" t="inlineStr">
-        <is>
-          <t>Andrew, Dov, Tanya</t>
-        </is>
-      </c>
-      <c r="D183" s="3" t="inlineStr">
-        <is>
-          <t>andrew@theandrewschulz.com</t>
-        </is>
-      </c>
-      <c r="E183" s="3" t="inlineStr">
-        <is>
-          <t>Cold outreach</t>
-        </is>
-      </c>
-      <c r="F183" s="3" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="G183" s="3" t="inlineStr">
-        <is>
-          <t>Cold — comedian target</t>
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>Agency Outreach — CAA / WME / UTA (individual agents, Feb–Mar 2026)</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>Schools — additional cold</t>
+          <t>Kevin Gelbard</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>College AD/coach</t>
+          <t>CAA</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>Holy Cross (Johnson/Paulsen/Rawlings), Stonehill (Kraus), UMBC (Lawson), Loyola (Blue), Coll. of Charleston (Harriman), Northeastern (Janning), BU (Quinn), UPenn</t>
+          <t>Agent</t>
         </is>
       </c>
       <c r="D184" s="3" t="inlineStr">
         <is>
-          <t>(various .edu)</t>
+          <t>kevin.gelbard@caa.com</t>
         </is>
       </c>
       <c r="E184" s="3" t="inlineStr">
         <is>
-          <t>Feb–Aug outreach</t>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
         </is>
       </c>
       <c r="F184" s="3" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="G184" s="3" t="inlineStr">
         <is>
-          <t>Mixed — BU responded; rest cold</t>
+          <t>RESPONDED — Ludacris/Tim McGraw; active</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
         <is>
-          <t>O'Melveny &amp; Myers</t>
+          <t>Peter Hess</t>
         </is>
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>Law firm</t>
+          <t>CAA</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>Aronson, Reinstein, Afner</t>
+          <t>Agent</t>
         </is>
       </c>
       <c r="D185" s="3" t="inlineStr">
         <is>
-          <t>baronson@omm.com</t>
+          <t>peter.hess@caa.com</t>
         </is>
       </c>
       <c r="E185" s="3" t="inlineStr">
         <is>
-          <t>Cold outreach</t>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
         </is>
       </c>
       <c r="F185" s="3" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="G185" s="3" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>RESPONDED — Colin Jost/Foxx/Teller/Cooper/Bateman/Fallon; revisit</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="3" t="inlineStr">
+        <is>
+          <t>Carla Laur</t>
+        </is>
+      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D186" s="3" t="inlineStr">
+        <is>
+          <t>claur@caa.com</t>
+        </is>
+      </c>
+      <c r="E186" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F186" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G186" s="3" t="inlineStr">
+        <is>
+          <t>RESPONDED — Miles Teller/Walton Goggins; revisit</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="3" t="inlineStr">
+        <is>
+          <t>Rick Lucas</t>
+        </is>
+      </c>
+      <c r="B187" s="3" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="C187" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D187" s="3" t="inlineStr">
+        <is>
+          <t>rlucas@caa.com</t>
+        </is>
+      </c>
+      <c r="E187" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F187" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G187" s="3" t="inlineStr">
+        <is>
+          <t>RESPONDED — Jamie Foxx; revisit</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="3" t="inlineStr">
+        <is>
+          <t>Adam Nettler</t>
+        </is>
+      </c>
+      <c r="B188" s="3" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D188" s="3" t="inlineStr">
+        <is>
+          <t>adam.nettler@caa.com</t>
+        </is>
+      </c>
+      <c r="E188" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F188" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G188" s="3" t="inlineStr">
+        <is>
+          <t>RESPONDED — unscripted TV; revisit</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="3" t="inlineStr">
+        <is>
+          <t>Matt Blake</t>
+        </is>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="C189" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D189" s="3" t="inlineStr">
+        <is>
+          <t>matt.blake@caa.com</t>
+        </is>
+      </c>
+      <c r="E189" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F189" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G189" s="3" t="inlineStr">
+        <is>
+          <t>RESPONDED — revisit</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="3" t="inlineStr">
+        <is>
+          <t>Landon Shepanek</t>
+        </is>
+      </c>
+      <c r="B190" s="3" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="C190" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D190" s="3" t="inlineStr">
+        <is>
+          <t>landon.shepanek@caa.com</t>
+        </is>
+      </c>
+      <c r="E190" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F190" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G190" s="3" t="inlineStr">
+        <is>
+          <t>RESPONDED — revisit</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="3" t="inlineStr">
+        <is>
+          <t>Bryan Lourd</t>
+        </is>
+      </c>
+      <c r="B191" s="3" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="C191" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D191" s="3" t="inlineStr">
+        <is>
+          <t>blourd@caa.com</t>
+        </is>
+      </c>
+      <c r="E191" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F191" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G191" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="3" t="inlineStr">
+        <is>
+          <t>Christian Carino</t>
+        </is>
+      </c>
+      <c r="B192" s="3" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D192" s="3" t="inlineStr">
+        <is>
+          <t>ccarino@caa.com</t>
+        </is>
+      </c>
+      <c r="E192" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F192" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G192" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="3" t="inlineStr">
+        <is>
+          <t>Rick Kurtzman</t>
+        </is>
+      </c>
+      <c r="B193" s="3" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="C193" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D193" s="3" t="inlineStr">
+        <is>
+          <t>rkurtzman@caa.com</t>
+        </is>
+      </c>
+      <c r="E193" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F193" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G193" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="3" t="inlineStr">
+        <is>
+          <t>Ethan Kurtzman</t>
+        </is>
+      </c>
+      <c r="B194" s="3" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="C194" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D194" s="3" t="inlineStr">
+        <is>
+          <t>ethan.kurtzman@caa.com</t>
+        </is>
+      </c>
+      <c r="E194" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F194" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G194" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="3" t="inlineStr">
+        <is>
+          <t>J. Darmody</t>
+        </is>
+      </c>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="C195" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D195" s="3" t="inlineStr">
+        <is>
+          <t>jdarmody@caa.com</t>
+        </is>
+      </c>
+      <c r="E195" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F195" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G195" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="3" t="inlineStr">
+        <is>
+          <t>John MacGregor</t>
+        </is>
+      </c>
+      <c r="B196" s="3" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="C196" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D196" s="3" t="inlineStr">
+        <is>
+          <t>john.macgregor@caa.com</t>
+        </is>
+      </c>
+      <c r="E196" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F196" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G196" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="3" t="inlineStr">
+        <is>
+          <t>T. Brennan</t>
+        </is>
+      </c>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D197" s="3" t="inlineStr">
+        <is>
+          <t>tbrennan@caa.com</t>
+        </is>
+      </c>
+      <c r="E197" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F197" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G197" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="3" t="inlineStr">
+        <is>
+          <t>Matt Wind</t>
+        </is>
+      </c>
+      <c r="B198" s="3" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D198" s="3" t="inlineStr">
+        <is>
+          <t>matt.wind@caa.com</t>
+        </is>
+      </c>
+      <c r="E198" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F198" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G198" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="3" t="inlineStr">
+        <is>
+          <t>Alex Douma</t>
+        </is>
+      </c>
+      <c r="B199" s="3" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="C199" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D199" s="3" t="inlineStr">
+        <is>
+          <t>alex.douma@caa.com</t>
+        </is>
+      </c>
+      <c r="E199" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F199" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G199" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="3" t="inlineStr">
+        <is>
+          <t>J. Lieberman</t>
+        </is>
+      </c>
+      <c r="B200" s="3" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D200" s="3" t="inlineStr">
+        <is>
+          <t>jlieberman@caa.com</t>
+        </is>
+      </c>
+      <c r="E200" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F200" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G200" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="3" t="inlineStr">
+        <is>
+          <t>Yale Jesser</t>
+        </is>
+      </c>
+      <c r="B201" s="3" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D201" s="3" t="inlineStr">
+        <is>
+          <t>yale.jesser@caa.com</t>
+        </is>
+      </c>
+      <c r="E201" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F201" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G201" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="3" t="inlineStr">
+        <is>
+          <t>David Sherman</t>
+        </is>
+      </c>
+      <c r="B202" s="3" t="inlineStr">
+        <is>
+          <t>WME (agency)</t>
+        </is>
+      </c>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D202" s="3" t="inlineStr">
+        <is>
+          <t>dsherman@wmeagency.com</t>
+        </is>
+      </c>
+      <c r="E202" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F202" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G202" s="3" t="inlineStr">
+        <is>
+          <t>RESPONDED — existing connection</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="3" t="inlineStr">
+        <is>
+          <t>M. Jasper</t>
+        </is>
+      </c>
+      <c r="B203" s="3" t="inlineStr">
+        <is>
+          <t>WME (agency)</t>
+        </is>
+      </c>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D203" s="3" t="inlineStr">
+        <is>
+          <t>mjasper@wmeagency.com</t>
+        </is>
+      </c>
+      <c r="E203" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F203" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G203" s="3" t="inlineStr">
+        <is>
+          <t>RESPONDED — revisit</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="3" t="inlineStr">
+        <is>
+          <t>T. Curtis</t>
+        </is>
+      </c>
+      <c r="B204" s="3" t="inlineStr">
+        <is>
+          <t>WME (agency)</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D204" s="3" t="inlineStr">
+        <is>
+          <t>tcurtis@wmeagency.com</t>
+        </is>
+      </c>
+      <c r="E204" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F204" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G204" s="3" t="inlineStr">
+        <is>
+          <t>RESPONDED — revisit</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="3" t="inlineStr">
+        <is>
+          <t>M. Rudman</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>WME (agency)</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D205" s="3" t="inlineStr">
+        <is>
+          <t>mrudman@wmeagency.com</t>
+        </is>
+      </c>
+      <c r="E205" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F205" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G205" s="3" t="inlineStr">
+        <is>
+          <t>RESPONDED — revisit</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="3" t="inlineStr">
+        <is>
+          <t>R. Koslowsky</t>
+        </is>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>WME (agency)</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D206" s="3" t="inlineStr">
+        <is>
+          <t>rkoslowsky@wmeagency.com</t>
+        </is>
+      </c>
+      <c r="E206" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F206" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G206" s="3" t="inlineStr">
+        <is>
+          <t>RESPONDED — revisit</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="3" t="inlineStr">
+        <is>
+          <t>DJS</t>
+        </is>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>WME (agency)</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D207" s="3" t="inlineStr">
+        <is>
+          <t>djs@wmeagency.com</t>
+        </is>
+      </c>
+      <c r="E207" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F207" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G207" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="3" t="inlineStr">
+        <is>
+          <t>JZH</t>
+        </is>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>WME (agency)</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D208" s="3" t="inlineStr">
+        <is>
+          <t>jzh@wmeagency.com</t>
+        </is>
+      </c>
+      <c r="E208" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F208" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G208" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="3" t="inlineStr">
+        <is>
+          <t>Andrew Mathes</t>
+        </is>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>WME (agency)</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D209" s="3" t="inlineStr">
+        <is>
+          <t>andrew.mathes@wmeagency.com</t>
+        </is>
+      </c>
+      <c r="E209" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F209" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G209" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="3" t="inlineStr">
+        <is>
+          <t>M. Maulitz</t>
+        </is>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>WME (agency)</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D210" s="3" t="inlineStr">
+        <is>
+          <t>mmaulitz@wmeagency.com</t>
+        </is>
+      </c>
+      <c r="E210" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F210" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G210" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="3" t="inlineStr">
+        <is>
+          <t>L. Buckley</t>
+        </is>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>WME (agency)</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D211" s="3" t="inlineStr">
+        <is>
+          <t>lbuckley@wmeagency.com</t>
+        </is>
+      </c>
+      <c r="E211" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F211" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G211" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="3" t="inlineStr">
+        <is>
+          <t>T. Jacobs</t>
+        </is>
+      </c>
+      <c r="B212" s="3" t="inlineStr">
+        <is>
+          <t>WME (agency)</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D212" s="3" t="inlineStr">
+        <is>
+          <t>tjacobs@wmeagency.com</t>
+        </is>
+      </c>
+      <c r="E212" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F212" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G212" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="3" t="inlineStr">
+        <is>
+          <t>S. Conover</t>
+        </is>
+      </c>
+      <c r="B213" s="3" t="inlineStr">
+        <is>
+          <t>WME (agency)</t>
+        </is>
+      </c>
+      <c r="C213" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D213" s="3" t="inlineStr">
+        <is>
+          <t>sconover@wmeagency.com</t>
+        </is>
+      </c>
+      <c r="E213" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F213" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G213" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="3" t="inlineStr">
+        <is>
+          <t>Ari Emanuel (WME CEO)</t>
+        </is>
+      </c>
+      <c r="B214" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C214" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D214" s="3" t="inlineStr">
+        <is>
+          <t>aemanuel@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E214" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F214" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G214" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="3" t="inlineStr">
+        <is>
+          <t>Tim Curtis</t>
+        </is>
+      </c>
+      <c r="B215" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C215" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D215" s="3" t="inlineStr">
+        <is>
+          <t>tcurtis@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E215" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F215" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G215" s="3" t="inlineStr">
+        <is>
+          <t>RESPONDED — offered BU to Carell/Krasinski</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="3" t="inlineStr">
+        <is>
+          <t>M. Berkowitz</t>
+        </is>
+      </c>
+      <c r="B216" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C216" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D216" s="3" t="inlineStr">
+        <is>
+          <t>mberkowitz@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E216" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F216" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G216" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="3" t="inlineStr">
+        <is>
+          <t>Henry Reisch</t>
+        </is>
+      </c>
+      <c r="B217" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C217" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D217" s="3" t="inlineStr">
+        <is>
+          <t>hreisch@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E217" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F217" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G217" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="3" t="inlineStr">
+        <is>
+          <t>Jeff Lesh</t>
+        </is>
+      </c>
+      <c r="B218" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C218" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D218" s="3" t="inlineStr">
+        <is>
+          <t>jlesh@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E218" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F218" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G218" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="3" t="inlineStr">
+        <is>
+          <t>Brad Slater</t>
+        </is>
+      </c>
+      <c r="B219" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D219" s="3" t="inlineStr">
+        <is>
+          <t>bslater@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E219" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F219" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G219" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="3" t="inlineStr">
+        <is>
+          <t>Danny Greenberg</t>
+        </is>
+      </c>
+      <c r="B220" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C220" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D220" s="3" t="inlineStr">
+        <is>
+          <t>dgreenberg@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E220" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F220" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G220" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="3" t="inlineStr">
+        <is>
+          <t>Nate Towne</t>
+        </is>
+      </c>
+      <c r="B221" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C221" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D221" s="3" t="inlineStr">
+        <is>
+          <t>ntowne@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E221" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F221" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G221" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="3" t="inlineStr">
+        <is>
+          <t>Joey Lee</t>
+        </is>
+      </c>
+      <c r="B222" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C222" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D222" s="3" t="inlineStr">
+        <is>
+          <t>leej@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E222" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F222" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G222" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="3" t="inlineStr">
+        <is>
+          <t>N. Josephson</t>
+        </is>
+      </c>
+      <c r="B223" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C223" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D223" s="3" t="inlineStr">
+        <is>
+          <t>njosephson@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E223" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F223" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G223" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="3" t="inlineStr">
+        <is>
+          <t>Andrew Finkelstein</t>
+        </is>
+      </c>
+      <c r="B224" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C224" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D224" s="3" t="inlineStr">
+        <is>
+          <t>afinkelstein@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E224" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F224" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G224" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="3" t="inlineStr">
+        <is>
+          <t>Douglas Edley</t>
+        </is>
+      </c>
+      <c r="B225" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C225" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D225" s="3" t="inlineStr">
+        <is>
+          <t>dedley@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E225" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F225" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G225" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="3" t="inlineStr">
+        <is>
+          <t>Kevin Dees</t>
+        </is>
+      </c>
+      <c r="B226" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C226" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D226" s="3" t="inlineStr">
+        <is>
+          <t>kdees@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E226" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F226" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G226" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="3" t="inlineStr">
+        <is>
+          <t>S. Mark</t>
+        </is>
+      </c>
+      <c r="B227" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C227" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D227" s="3" t="inlineStr">
+        <is>
+          <t>smark@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E227" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F227" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G227" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="3" t="inlineStr">
+        <is>
+          <t>W. Lowery</t>
+        </is>
+      </c>
+      <c r="B228" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C228" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D228" s="3" t="inlineStr">
+        <is>
+          <t>wlowery@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E228" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F228" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G228" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="3" t="inlineStr">
+        <is>
+          <t>W. Zavala</t>
+        </is>
+      </c>
+      <c r="B229" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C229" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D229" s="3" t="inlineStr">
+        <is>
+          <t>wzavala@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E229" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F229" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G229" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="3" t="inlineStr">
+        <is>
+          <t>N. Hoagland</t>
+        </is>
+      </c>
+      <c r="B230" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C230" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D230" s="3" t="inlineStr">
+        <is>
+          <t>nhoagland@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E230" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F230" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G230" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="3" t="inlineStr">
+        <is>
+          <t>D. Lucterhand</t>
+        </is>
+      </c>
+      <c r="B231" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C231" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D231" s="3" t="inlineStr">
+        <is>
+          <t>dlucterhand@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E231" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F231" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G231" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="3" t="inlineStr">
+        <is>
+          <t>D. Becky</t>
+        </is>
+      </c>
+      <c r="B232" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C232" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D232" s="3" t="inlineStr">
+        <is>
+          <t>dbecky@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E232" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F232" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G232" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="3" t="inlineStr">
+        <is>
+          <t>D. Levine</t>
+        </is>
+      </c>
+      <c r="B233" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C233" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D233" s="3" t="inlineStr">
+        <is>
+          <t>dlevine@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E233" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F233" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G233" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="3" t="inlineStr">
+        <is>
+          <t>J. Kovacevic</t>
+        </is>
+      </c>
+      <c r="B234" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C234" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D234" s="3" t="inlineStr">
+        <is>
+          <t>jkovacevic@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E234" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F234" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G234" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="3" t="inlineStr">
+        <is>
+          <t>J. Thomas</t>
+        </is>
+      </c>
+      <c r="B235" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C235" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D235" s="3" t="inlineStr">
+        <is>
+          <t>jthomas@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E235" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F235" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G235" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="3" t="inlineStr">
+        <is>
+          <t>K. Sarkisian</t>
+        </is>
+      </c>
+      <c r="B236" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C236" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D236" s="3" t="inlineStr">
+        <is>
+          <t>ksarkisian@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E236" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F236" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G236" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="3" t="inlineStr">
+        <is>
+          <t>T. Bernardy</t>
+        </is>
+      </c>
+      <c r="B237" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C237" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D237" s="3" t="inlineStr">
+        <is>
+          <t>tbernardy@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E237" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F237" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G237" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="3" t="inlineStr">
+        <is>
+          <t>R. Rosen</t>
+        </is>
+      </c>
+      <c r="B238" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C238" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D238" s="3" t="inlineStr">
+        <is>
+          <t>rrosen@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E238" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F238" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G238" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="3" t="inlineStr">
+        <is>
+          <t>J. Williams</t>
+        </is>
+      </c>
+      <c r="B239" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C239" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D239" s="3" t="inlineStr">
+        <is>
+          <t>jwilliams@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E239" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F239" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G239" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="3" t="inlineStr">
+        <is>
+          <t>J. Dixon</t>
+        </is>
+      </c>
+      <c r="B240" s="3" t="inlineStr">
+        <is>
+          <t>WME Ent</t>
+        </is>
+      </c>
+      <c r="C240" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D240" s="3" t="inlineStr">
+        <is>
+          <t>jdixon@wmeentertainment.com</t>
+        </is>
+      </c>
+      <c r="E240" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F240" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G240" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="3" t="inlineStr">
+        <is>
+          <t>K. Volchok</t>
+        </is>
+      </c>
+      <c r="B241" s="3" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="C241" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D241" s="3" t="inlineStr">
+        <is>
+          <t>volchokk@unitedtalent.com</t>
+        </is>
+      </c>
+      <c r="E241" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F241" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G241" s="3" t="inlineStr">
+        <is>
+          <t>RESPONDED — revisit</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="3" t="inlineStr">
+        <is>
+          <t>R. Klubeck</t>
+        </is>
+      </c>
+      <c r="B242" s="3" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="C242" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D242" s="3" t="inlineStr">
+        <is>
+          <t>klubeckr@unitedtalent.com</t>
+        </is>
+      </c>
+      <c r="E242" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F242" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G242" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="3" t="inlineStr">
+        <is>
+          <t>Brett Duchon</t>
+        </is>
+      </c>
+      <c r="B243" s="3" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="C243" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D243" s="3" t="inlineStr">
+        <is>
+          <t>duchonb@unitedtalent.com</t>
+        </is>
+      </c>
+      <c r="E243" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F243" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G243" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="3" t="inlineStr">
+        <is>
+          <t>Bill Lazarus</t>
+        </is>
+      </c>
+      <c r="B244" s="3" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="C244" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D244" s="3" t="inlineStr">
+        <is>
+          <t>lazarusb@unitedtalent.com</t>
+        </is>
+      </c>
+      <c r="E244" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F244" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G244" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="3" t="inlineStr">
+        <is>
+          <t>Nancy Gates</t>
+        </is>
+      </c>
+      <c r="B245" s="3" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="C245" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D245" s="3" t="inlineStr">
+        <is>
+          <t>gatesn@unitedtalent.com</t>
+        </is>
+      </c>
+      <c r="E245" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F245" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G245" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="3" t="inlineStr">
+        <is>
+          <t>Jeremy Barber</t>
+        </is>
+      </c>
+      <c r="B246" s="3" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="C246" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D246" s="3" t="inlineStr">
+        <is>
+          <t>barberj@unitedtalent.com</t>
+        </is>
+      </c>
+      <c r="E246" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F246" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G246" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="3" t="inlineStr">
+        <is>
+          <t>Jason Heyman</t>
+        </is>
+      </c>
+      <c r="B247" s="3" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="C247" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D247" s="3" t="inlineStr">
+        <is>
+          <t>heymanj@unitedtalent.com</t>
+        </is>
+      </c>
+      <c r="E247" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F247" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G247" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="3" t="inlineStr">
+        <is>
+          <t>Jacob Lawson</t>
+        </is>
+      </c>
+      <c r="B248" s="3" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="C248" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D248" s="3" t="inlineStr">
+        <is>
+          <t>lawsonj@unitedtalent.com</t>
+        </is>
+      </c>
+      <c r="E248" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F248" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G248" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="3" t="inlineStr">
+        <is>
+          <t>Greg Janes</t>
+        </is>
+      </c>
+      <c r="B249" s="3" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="C249" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D249" s="3" t="inlineStr">
+        <is>
+          <t>janeseg@unitedtalent.com</t>
+        </is>
+      </c>
+      <c r="E249" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F249" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G249" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="3" t="inlineStr">
+        <is>
+          <t>Babbette Perry</t>
+        </is>
+      </c>
+      <c r="B250" s="3" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="C250" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D250" s="3" t="inlineStr">
+        <is>
+          <t>perryb@unitedtalent.com</t>
+        </is>
+      </c>
+      <c r="E250" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F250" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G250" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="3" t="inlineStr">
+        <is>
+          <t>John Sacks</t>
+        </is>
+      </c>
+      <c r="B251" s="3" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="C251" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D251" s="3" t="inlineStr">
+        <is>
+          <t>sacksj@unitedtalent.com</t>
+        </is>
+      </c>
+      <c r="E251" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F251" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G251" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="3" t="inlineStr">
+        <is>
+          <t>N. Nuciforo</t>
+        </is>
+      </c>
+      <c r="B252" s="3" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="C252" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D252" s="3" t="inlineStr">
+        <is>
+          <t>nuciforon@unitedtalent.com</t>
+        </is>
+      </c>
+      <c r="E252" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F252" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G252" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="3" t="inlineStr">
+        <is>
+          <t>B. Balbo</t>
+        </is>
+      </c>
+      <c r="B253" s="3" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="C253" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D253" s="3" t="inlineStr">
+        <is>
+          <t>balbob@unitedtalent.com</t>
+        </is>
+      </c>
+      <c r="E253" s="3" t="inlineStr">
+        <is>
+          <t>Feb–Mar 2026 cold outreach ('NCAA Acquisition + Production')</t>
+        </is>
+      </c>
+      <c r="F253" s="3" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="G253" s="3" t="inlineStr">
+        <is>
+          <t>Cold — sent, no reply</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A123:G123"/>
     <mergeCell ref="A141:G141"/>
     <mergeCell ref="A97:G97"/>
     <mergeCell ref="A79:G79"/>
     <mergeCell ref="A55:G55"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A183:G183"/>
     <mergeCell ref="A10:G10"/>
     <mergeCell ref="A133:G133"/>
   </mergeCells>

</xml_diff>

<commit_message>
Replace celebrity target list with authoritative Making Cinderella 'targets' tab
Implements the robust targets list from the Making Cinderella Google Sheet:
5-column School / Lead / Co-Lead / Co-Lead / Status layout (66 rows),
replacing the prior 4-column shortlist. Adds schools-without-leads as
candidate rows and carries status signal where known.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ajJRqKa1DUy4iKHJKPEi3
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-08-12-cinderella-contacts.xlsx
+++ b/cinderella/Outputs/2026-08-12-cinderella-contacts.xlsx
@@ -9543,13 +9543,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9560,15 +9561,20 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Celebrity option(s)</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Co-Lead</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Co-Lead</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -9587,256 +9593,272 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Alum / attached (Unanimous)</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>ATTACHED — flagship</t>
+          <t>Ryan Reynolds</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>ATTACHED — flagship; LOI signed</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Saint Joseph's</t>
+          <t>New Hampshire</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Kevin Hart, Bradley Cooper, Jason Kelce, Charles Barkley, Will Smith</t>
+          <t>Adam Sandler</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Philly (regional)</t>
+          <t>Triple H</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>LOI signed; celeb TBD (Hart active)</t>
+          <t>Seth Meyers</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>LOI in play (Sandler via Happy Madison)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Tulane</t>
+          <t>Fordham</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Woody Harrelson (+ Simu Liu)</t>
+          <t>Denzel Washington</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Film hook (WMCJ)</t>
+          <t>Mike Breen</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>TOP TARGET — warm via Simu</t>
+          <t>Chaz Palminteri</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Verified alumni (Denzel, Breen)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Merrimack / Vermont / Northeastern</t>
+          <t>Northeastern</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Ben Affleck</t>
+          <t>Mark Wahlberg</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Boston-regional</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Engaging</t>
-        </is>
-      </c>
+          <t>Bill Burr</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>New Hampshire</t>
+          <t>George Washington</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Adam Sandler, Triple H, Seth Meyers</t>
+          <t>Dave Chappelle</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Regional</t>
+          <t>Pharrell Williams</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>LOI in play (Sandler via Happy Madison)</t>
+          <t>Casey Affleck</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Met 8/7 (Caputo/Lipitz) — active</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Fordham</t>
+          <t>Loyola Chicago</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Denzel Washington, Mike Breen</t>
+          <t>Barack Obama</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Verified alumni + hoops</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>On-thesis</t>
-        </is>
-      </c>
+          <t>Tim Grover</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Indiana State</t>
+          <t>Merrimack</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Larry Bird, David Goggins</t>
+          <t>Ben Affleck</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Bird alum; Goggins geo</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>PMG roster</t>
+          <t>Charlie Day</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Call Aug 19 — active</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Central Arkansas</t>
+          <t>St. Joseph's</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Scottie Pippen (+ Clinton/Thornton)</t>
+          <t>Kevin Hart</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Alum</t>
+          <t>Bradley Cooper</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>PMG roster</t>
+          <t>Jason Kelce</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>LOI SIGNED — celeb TBD (Hart active)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Southern Illinois</t>
+          <t>Boston College</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Walt 'Clyde' Frazier (+ McCarthy/Odenkirk)</t>
+          <t>Chris Evans</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>All SIU alumni</t>
+          <t>John Krasinski</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>PMG (Frazier) — strong pairing</t>
+          <t>BJ Novak</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Fallen-giant track</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>UMass</t>
+          <t>UMKC</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Julius Erving (+ Richard Gere)</t>
+          <t>Jason Sudeikis</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Alumni</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>PMG (Erving); Dr. J also Philly</t>
-        </is>
-      </c>
+          <t>Paul Rudd</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>UTEP</t>
+          <t>Hawaii</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Tim Hardaway (+ Glory Road)</t>
+          <t>Dwayne Johnson</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Alum</t>
+          <t>Bruno Mars</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>PMG roster</t>
-        </is>
-      </c>
+          <t>Jason Momoa</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Furman</t>
+          <t>Belmont</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Kevin Garnett</t>
+          <t>Justin Timberlake</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>HS ~20 min away</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Idea (per email)</t>
-        </is>
-      </c>
+          <t>Brad Paisley</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -9851,166 +9873,1076 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Verified alum</t>
+          <t>John A. Sobrato</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Via CTRL / WME</t>
+          <t>Jaylen Williams</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Nash via CTRL / WME</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Boston College</t>
+          <t>Holy Cross</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Bill Murray (via son Luke, HC), Amy Poehler</t>
+          <t>Bill Simmons</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>BC ties</t>
+          <t>Conan O'Brien</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Fallen-giant track</t>
-        </is>
-      </c>
+          <t>Denis Leary</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Wake Forest</t>
+          <t>Boston University</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Tim Duncan, Muggsy Bogues</t>
+          <t>Ben Affleck</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Verified Deacons</t>
+          <t>Matt Damon</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Fallen-giant track</t>
+          <t>Jason Alexander</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>(WME/Tim Curtis floated Carell + Krasinski)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>NYU (D3)</t>
+          <t>UC Irvine</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Adam Sandler, Billy Crystal, Spike Lee</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Verified Tisch alumni</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>D3 track</t>
-        </is>
-      </c>
+          <t>Will Ferrell</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Johns Hopkins (D3)</t>
+          <t>UC Santa Barbara</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Mike Bloomberg, Michael Phelps, Carmelo Anthony</t>
+          <t>Andrew Schulz</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Alum/local</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>D3 track</t>
+          <t>Michael Douglas</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Schulz camp contacted</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Ivy outreach</t>
+          <t>LIU</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Yale, Brown, Harvard staff contacted</t>
+          <t>Jay-Z</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Billy Joel</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Exploratory</t>
-        </is>
-      </c>
+          <t>Ray Dalio</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Reps in motion</t>
+          <t>Tulane</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Ludacris &amp; Tim McGraw (CAA/Gelbard); Brian Scalabrine (direct)</t>
+          <t>The Mannings</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Theo Von</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Agent pass-through active</t>
+          <t>Anthony Mackie</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>TOP TARGET — also Woody Harrelson (via Simu Liu)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Via CAA (Peter Hess / Carla Laur / Rick Lucas)</t>
+          <t>Temple</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Colin Jost, Jamie Foxx, Miles Teller, Walton Goggins, Bradley Cooper</t>
+          <t>Kevin Hart</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>CAA-repped</t>
+          <t>Adam McKay</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Offers made Mar 2026 — outstanding; revisit</t>
+          <t>Judd Apatow</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>(Hart moved to St. Joe's per vault)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>North Texas</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Jamie Foxx</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Post Malone</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Steve Austin</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Foxx via CAA / Rick Lucas</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Detroit</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Keegan-Michael Key</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Eminem</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Charleston</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Bill Murray</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Danny McBride</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Darius Rucker</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Murray = RiverDogs co-owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Justin Bieber</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Dave Burd</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Elon</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Shane Gillis</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Chris Daughtry</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Daughtry≠Elon (verify)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Rhode Island</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Seth MacFarlane</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Charlie Day</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Jay Leno</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Leno≠URI (verify)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>UMass</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>John Cena</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Liev Schreiber</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Cena=Springfield(D3); Schreiber≠UMass (verify)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Appalachian State</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Eric Church</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Luke Combs</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>William &amp; Mary</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Jon Stewart</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Todd Boehly</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Lehigh</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>CJ McCollum</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Dwayne Johnson</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Northern Illinois</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Vince Vaughn</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Sebastian Maniscalco</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Ball State</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>David Letterman</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Jim Nantz</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Letterman verified; Nantz≠Ball State (verify)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Drake</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Jeremy Piven</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Zach Johnson</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Cal State Fullerton</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Kevin Costner</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Will Ferrell</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Steve Martin</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Texas Southern</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Michael Strahan</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Travis Scott</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Kent State</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Steve Harvey</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Michael Keaton</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Georgia Southern</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Walton Goggins</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Luke Bryan</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Druski</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Goggins via CAA / Carla Laur</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Georgia State</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Ludacris</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Gucci Mane</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Luda via CAA / Gelbard</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Marshall</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Billy Crystal</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>O.J. Mayo</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr"/>
+      <c r="E40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Missouri State</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Brad Pitt</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>John Goodman</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>New Orleans</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Theo Von</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Anthony Mackie</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr"/>
+      <c r="E42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Texas State</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Taylor Sheridan</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Shawn Michaels</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Wichita State</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Paul Wight</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Antoine Carr</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr"/>
+      <c r="E44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Oregon State</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Gary Payton</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Indiana State</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Larry Bird</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>John Mellencamp</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr"/>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Bird/Goggins via PMG</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Louisiana Monroe</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Tim McGraw</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>McGraw via CAA / Gelbard</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>UTEP</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Tim Hardaway</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr"/>
+      <c r="D48" s="3" t="inlineStr"/>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>PMG roster</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Central Arkansas</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Scottie Pippen</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>PMG roster</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Saint Louis</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Larry Hughes</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Jayson Tatum</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr"/>
+      <c r="E50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Tennessee State</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Oprah Winfrey</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr"/>
+      <c r="E51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Stanford</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Tiger Woods</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>John McEnroe</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr"/>
+      <c r="E52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>USC</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Will Ferrell</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Brian Scalabrine</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr"/>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Scalabrine direct-contacted</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>South Carolina</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Darius Rucker</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr"/>
+      <c r="D54" s="3" t="inlineStr"/>
+      <c r="E54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Wake Forest</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Tim Duncan</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Muggsy Bogues</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr"/>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Verified Deacons</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Providence</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Seth MacFarlane</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Doris Burke</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr"/>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Burke verified alum</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>Hofstra</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Jerry Seinfeld</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Christopher Walken</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr"/>
+      <c r="E57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>ETSU</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Kenny Chesney</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr"/>
+      <c r="D58" s="3" t="inlineStr"/>
+      <c r="E58" s="3" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Fairfield</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>John Mayer</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr"/>
+      <c r="D59" s="3" t="inlineStr"/>
+      <c r="E59" s="3" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Furman</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Clint Dempsey</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr"/>
+      <c r="D60" s="3" t="inlineStr"/>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>(Garnett HS nearby — prior note)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr"/>
+      <c r="C61" s="3" t="inlineStr"/>
+      <c r="D61" s="3" t="inlineStr"/>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>School candidate — no lead yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>High Point</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr"/>
+      <c r="C62" s="3" t="inlineStr"/>
+      <c r="D62" s="3" t="inlineStr"/>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>School candidate — no lead yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Loyola Marymount</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr"/>
+      <c r="C63" s="3" t="inlineStr"/>
+      <c r="D63" s="3" t="inlineStr"/>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>School candidate — no lead yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>VCU</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr"/>
+      <c r="C64" s="3" t="inlineStr"/>
+      <c r="D64" s="3" t="inlineStr"/>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>School candidate — no lead yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>UNC Greensboro</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr"/>
+      <c r="C65" s="3" t="inlineStr"/>
+      <c r="D65" s="3" t="inlineStr"/>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>School candidate — no lead yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>Denver</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr"/>
+      <c r="C66" s="3" t="inlineStr"/>
+      <c r="D66" s="3" t="inlineStr"/>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>School candidate — no lead yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>Pepperdine</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr"/>
+      <c r="C67" s="3" t="inlineStr"/>
+      <c r="D67" s="3" t="inlineStr"/>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>School candidate — no lead yet</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Kevin Garnett to Furman; add 3 suggested-fit candidates per school
- Furman: add Kevin Garnett as co-lead (Mauldin/Greenville SC regional tie).
- Celebrity Targets: three new 'Suggested Fit' columns per school with
  Claude-added candidates (alum or regional/adopted-city), all flagged for
  tie verification before external use.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ajJRqKa1DUy4iKHJKPEi3
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-08-12-cinderella-contacts.xlsx
+++ b/cinderella/Outputs/2026-08-12-cinderella-contacts.xlsx
@@ -12,6 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Contacts'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Celebrity Targets'!$A$1:$H$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -82,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -91,7 +92,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -9543,38 +9543,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>School</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Lead</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Co-Lead</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Co-Lead</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Suggested Fit 1</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Suggested Fit 2</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Suggested Fit 3</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -9599,6 +9617,21 @@
       <c r="D2" s="3" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr">
         <is>
+          <t>J. Cole</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Michael Jordan</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Anthony Foxx</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
           <t>ATTACHED — flagship; LOI signed</t>
         </is>
       </c>
@@ -9626,6 +9659,21 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
+          <t>Sarah Silverman</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Bode Miller</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Dan Brown</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
           <t>LOI in play (Sandler via Happy Madison)</t>
         </is>
       </c>
@@ -9653,6 +9701,21 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
+          <t>Lana Del Rey</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Alan Alda</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Dylan McDermott</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
           <t>Verified alumni (Denzel, Breen)</t>
         </is>
       </c>
@@ -9674,7 +9737,22 @@
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Donnie Wahlberg</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Steve Carell</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Uzo Aduba</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -9699,6 +9777,21 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
+          <t>Kerry Washington</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Alec Baldwin</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Dave Grohl</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
           <t>Met 8/7 (Caputo/Lipitz) — active</t>
         </is>
       </c>
@@ -9720,7 +9813,22 @@
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Bob Newhart</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Dwyane Wade</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Chance the Rapper</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -9741,6 +9849,21 @@
       <c r="D8" s="3" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr">
         <is>
+          <t>Michael Chiklis</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Dane Cook</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Lenny Clarke</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
           <t>Call Aug 19 — active</t>
         </is>
       </c>
@@ -9768,6 +9891,21 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
+          <t>Will Smith</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Tina Fey</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Kevin Bacon</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
           <t>LOI SIGNED — celeb TBD (Hart active)</t>
         </is>
       </c>
@@ -9795,6 +9933,21 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
+          <t>Amy Poehler</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Doug Flutie</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Chris O'Donnell</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
           <t>Fallen-giant track</t>
         </is>
       </c>
@@ -9816,7 +9969,22 @@
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Eric Stonestreet</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Rob Riggle</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Janelle Monáe</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -9839,7 +10007,22 @@
           <t>Jason Momoa</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Nicole Scherzinger</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Marcus Mariota</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Bethany Hamilton</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -9858,7 +10041,22 @@
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Trisha Yearwood</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Reese Witherspoon</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Florida Georgia Line</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -9883,6 +10081,21 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
+          <t>Brandi Chastain</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Steve Kerr</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Aisha Tyler</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
           <t>Nash via CTRL / WME</t>
         </is>
       </c>
@@ -9908,7 +10121,22 @@
           <t>Denis Leary</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Bob Cousy</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Tommy Heinsohn</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Chris Matthews</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -9933,6 +10161,21 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
+          <t>Howard Stern</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Geena Davis</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Julianne Moore</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
           <t>(WME/Tim Curtis floated Carell + Krasinski)</t>
         </is>
       </c>
@@ -9950,7 +10193,22 @@
       </c>
       <c r="C17" s="3" t="inlineStr"/>
       <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Jon Lovitz</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Gwen Stefani</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Mark McGrath</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -9971,6 +10229,21 @@
       <c r="D18" s="3" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr">
         <is>
+          <t>Katy Perry</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Jack Johnson</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Rob Lowe</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
           <t>Schulz camp contacted</t>
         </is>
       </c>
@@ -9996,7 +10269,22 @@
           <t>Ray Dalio</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Rosie Perez</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Michael Rapaport</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Mike Tyson</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -10021,6 +10309,21 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
+          <t>Harry Connick Jr.</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Lil Wayne</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Wendell Pierce</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
           <t>TOP TARGET — also Woody Harrelson (via Simu Liu)</t>
         </is>
       </c>
@@ -10048,6 +10351,21 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
+          <t>Bob Saget</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Questlove</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Boyz II Men</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
           <t>(Hart moved to St. Joe's per vault)</t>
         </is>
       </c>
@@ -10075,6 +10393,21 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
+          <t>Don Henley</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Norah Jones</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Roy Orbison</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
           <t>Foxx via CAA / Rick Lucas</t>
         </is>
       </c>
@@ -10096,7 +10429,22 @@
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Big Sean</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Jack White</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Lily Tomlin</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -10121,6 +10469,21 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
+          <t>Stephen Colbert</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Thomas Gibson</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Shepard Fairey</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
           <t>Murray = RiverDogs co-owner</t>
         </is>
       </c>
@@ -10142,7 +10505,22 @@
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Jason Mraz</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Shirley MacLaine</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Warren Beatty</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -10163,6 +10541,21 @@
       <c r="D26" s="3" t="inlineStr"/>
       <c r="E26" s="3" t="inlineStr">
         <is>
+          <t>Ben Folds</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Evan Rachel Wood</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Emily Procter</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
           <t>Daughtry≠Elon (verify)</t>
         </is>
       </c>
@@ -10190,6 +10583,21 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
+          <t>Viola Davis</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>James Woods</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Debra Messing</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
           <t>Leno≠URI (verify)</t>
         </is>
       </c>
@@ -10213,6 +10621,21 @@
       <c r="D28" s="3" t="inlineStr"/>
       <c r="E28" s="3" t="inlineStr">
         <is>
+          <t>Julius Erving</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Richard Gere</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Jack Welch</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
           <t>Cena=Springfield(D3); Schreiber≠UMass (verify)</t>
         </is>
       </c>
@@ -10234,7 +10657,22 @@
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Zach Galifianakis</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Ric Flair</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Kellie Pickler</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -10253,7 +10691,22 @@
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr"/>
-      <c r="E30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Glenn Close</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Mike Tomlin</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Bruce Hornsby</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -10272,7 +10725,22 @@
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Amanda Seyfried</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Christine Taylor</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Daniel Roebuck</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -10291,7 +10759,22 @@
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr"/>
-      <c r="E32" s="3" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Dan Castellaneta</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Joan Allen</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>John C. Reilly</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -10312,6 +10795,21 @@
       <c r="D33" s="3" t="inlineStr"/>
       <c r="E33" s="3" t="inlineStr">
         <is>
+          <t>Jim Davis</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Joyce DeWitt</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Axl Rose</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
           <t>Letterman verified; Nantz≠Ball State (verify)</t>
         </is>
       </c>
@@ -10333,7 +10831,22 @@
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr"/>
-      <c r="E34" s="3" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Ashton Kutcher</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Elijah Wood</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Tom Arnold</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -10356,7 +10869,22 @@
           <t>Steve Martin</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Adam Carolla</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Snoop Dogg</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Jack Black</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -10375,7 +10903,22 @@
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr"/>
-      <c r="E36" s="3" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Megan Thee Stallion</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Beyoncé</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Lizzo</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -10394,7 +10937,22 @@
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Arsenio Hall</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Chrissie Hynde</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Joe Walsh</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -10419,6 +10977,21 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
+          <t>Jason Aldean</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Alan Jackson</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Killer Mike</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
           <t>Goggins via CAA / Carla Laur</t>
         </is>
       </c>
@@ -10442,6 +11015,21 @@
       <c r="D39" s="3" t="inlineStr"/>
       <c r="E39" s="3" t="inlineStr">
         <is>
+          <t>Usher</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Tyler Perry</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Jermaine Dupri</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
           <t>Luda via CAA / Gelbard</t>
         </is>
       </c>
@@ -10463,7 +11051,22 @@
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr"/>
-      <c r="E40" s="3" t="inlineStr"/>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Randy Moss</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Jason Williams</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>Jennifer Garner</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -10482,7 +11085,22 @@
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr"/>
-      <c r="E41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Kathleen Turner</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Sheryl Crow</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Jon Hamm</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -10501,7 +11119,22 @@
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr"/>
-      <c r="E42" s="3" t="inlineStr"/>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Master P</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Ellen DeGeneres</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>Trombone Shorty</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -10520,7 +11153,22 @@
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr"/>
-      <c r="E43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>George Strait</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Willie Nelson</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Matthew McConaughey</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -10539,7 +11187,22 @@
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr"/>
-      <c r="E44" s="3" t="inlineStr"/>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Xavier McDaniel</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Barry Sanders</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Cliff Levingston</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -10554,7 +11217,22 @@
       </c>
       <c r="C45" s="3" t="inlineStr"/>
       <c r="D45" s="3" t="inlineStr"/>
-      <c r="E45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>A.C. Green</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Danny Ainge</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>Ty Burrell</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -10574,6 +11252,21 @@
       </c>
       <c r="D46" s="3" t="inlineStr"/>
       <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Oscar Robertson</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>Adam Driver</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>Babyface</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
         <is>
           <t>Bird/Goggins via PMG</t>
         </is>
@@ -10594,6 +11287,21 @@
       <c r="D47" s="3" t="inlineStr"/>
       <c r="E47" s="3" t="inlineStr">
         <is>
+          <t>Kix Brooks</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Hunter Hayes</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Faith Hill</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
           <t>McGraw via CAA / Gelbard</t>
         </is>
       </c>
@@ -10613,6 +11321,21 @@
       <c r="D48" s="3" t="inlineStr"/>
       <c r="E48" s="3" t="inlineStr">
         <is>
+          <t>Khalid</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Nate Archibald</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Aaron Jones</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
           <t>PMG roster</t>
         </is>
       </c>
@@ -10632,6 +11355,21 @@
       <c r="D49" s="3" t="inlineStr"/>
       <c r="E49" s="3" t="inlineStr">
         <is>
+          <t>Kris Allen</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Billy Bob Thornton</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Mary Steenburgen</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
           <t>PMG roster</t>
         </is>
       </c>
@@ -10653,7 +11391,22 @@
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr"/>
-      <c r="E50" s="3" t="inlineStr"/>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Nelly</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Bradley Beal</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Jenna Fischer</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -10668,7 +11421,22 @@
       </c>
       <c r="C51" s="3" t="inlineStr"/>
       <c r="D51" s="3" t="inlineStr"/>
-      <c r="E51" s="3" t="inlineStr"/>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Miley Cyrus</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Kane Brown</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>CeCe Winans</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -10687,7 +11455,22 @@
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr"/>
-      <c r="E52" s="3" t="inlineStr"/>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>John Elway</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Sigourney Weaver</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Andrew Luck</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -10708,6 +11491,21 @@
       <c r="D53" s="3" t="inlineStr"/>
       <c r="E53" s="3" t="inlineStr">
         <is>
+          <t>George Lucas</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Forest Whitaker</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>America Ferrera</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
           <t>Scalabrine direct-contacted</t>
         </is>
       </c>
@@ -10725,7 +11523,22 @@
       </c>
       <c r="C54" s="3" t="inlineStr"/>
       <c r="D54" s="3" t="inlineStr"/>
-      <c r="E54" s="3" t="inlineStr"/>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Aziz Ansari</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Chris Rock</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Leeza Gibbons</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -10746,6 +11559,21 @@
       <c r="D55" s="3" t="inlineStr"/>
       <c r="E55" s="3" t="inlineStr">
         <is>
+          <t>Chris Paul</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Arnold Palmer</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>Josh Howard</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
           <t>Verified Deacons</t>
         </is>
       </c>
@@ -10769,6 +11597,21 @@
       <c r="D56" s="3" t="inlineStr"/>
       <c r="E56" s="3" t="inlineStr">
         <is>
+          <t>Ernie DiGregorio</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>God Shammgod</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>Peter Farrelly</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
           <t>Burke verified alum</t>
         </is>
       </c>
@@ -10790,7 +11633,22 @@
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr"/>
-      <c r="E57" s="3" t="inlineStr"/>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Francis Ford Coppola</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>James Caan</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>Susan Lucci</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -10805,7 +11663,22 @@
       </c>
       <c r="C58" s="3" t="inlineStr"/>
       <c r="D58" s="3" t="inlineStr"/>
-      <c r="E58" s="3" t="inlineStr"/>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Dolly Parton</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>Morgan Wallen</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>Keith Jennings</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -10820,7 +11693,22 @@
       </c>
       <c r="C59" s="3" t="inlineStr"/>
       <c r="D59" s="3" t="inlineStr"/>
-      <c r="E59" s="3" t="inlineStr"/>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Meg Ryan</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>Vince McMahon</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>Christopher Lloyd</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -10833,11 +11721,30 @@
           <t>Clint Dempsey</t>
         </is>
       </c>
-      <c r="C60" s="3" t="inlineStr"/>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Kevin Garnett</t>
+        </is>
+      </c>
       <c r="D60" s="3" t="inlineStr"/>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>(Garnett HS nearby — prior note)</t>
+          <t>Peabo Bryson</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>Marcus Lattimore</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>Keith Lockhart</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>KG = Mauldin/Greenville SC regional</t>
         </is>
       </c>
     </row>
@@ -10852,6 +11759,21 @@
       <c r="D61" s="3" t="inlineStr"/>
       <c r="E61" s="3" t="inlineStr">
         <is>
+          <t>Bill Walton</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>Tony Hawk</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>Cameron Diaz</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
           <t>School candidate — no lead yet</t>
         </is>
       </c>
@@ -10867,6 +11789,21 @@
       <c r="D62" s="3" t="inlineStr"/>
       <c r="E62" s="3" t="inlineStr">
         <is>
+          <t>Fantasia Barrino</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>Rhiannon Giddens</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>Randy Travis</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
           <t>School candidate — no lead yet</t>
         </is>
       </c>
@@ -10882,6 +11819,21 @@
       <c r="D63" s="3" t="inlineStr"/>
       <c r="E63" s="3" t="inlineStr">
         <is>
+          <t>Colin Hanks</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>Bo Kimble</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>Brooke Burke</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
           <t>School candidate — no lead yet</t>
         </is>
       </c>
@@ -10897,6 +11849,21 @@
       <c r="D64" s="3" t="inlineStr"/>
       <c r="E64" s="3" t="inlineStr">
         <is>
+          <t>D'Angelo</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>Missy Elliott</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>Timbaland</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
           <t>School candidate — no lead yet</t>
         </is>
       </c>
@@ -10912,6 +11879,21 @@
       <c r="D65" s="3" t="inlineStr"/>
       <c r="E65" s="3" t="inlineStr">
         <is>
+          <t>Warren Haynes</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Petey Pablo</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>Clay Aiken</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
           <t>School candidate — no lead yet</t>
         </is>
       </c>
@@ -10927,6 +11909,21 @@
       <c r="D66" s="3" t="inlineStr"/>
       <c r="E66" s="3" t="inlineStr">
         <is>
+          <t>Chauncey Billups</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>Tim Allen</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>Trey Parker</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
           <t>School candidate — no lead yet</t>
         </is>
       </c>
@@ -10942,11 +11939,27 @@
       <c r="D67" s="3" t="inlineStr"/>
       <c r="E67" s="3" t="inlineStr">
         <is>
+          <t>Doug Christie</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Dick Van Dyke</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>Pierce Brosnan</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
           <t>School candidate — no lead yet</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix targets: remove deceased suggestions and drop bad Leno/URI tie
- Remove Jay Leno from Rhode Island (no RI tie; Andover MA / LA).
- Replace 8 deceased names with living, same-tie alternatives:
  Walton->Mario Lopez (San Diego), Newhart->Common (Chicago),
  Heinsohn->Billy Collins (Holy Cross), Orbison->Erykah Badu (N. Texas),
  Welch->Marcus Camby (UMass hoops), Palmer->Webb Simpson (Wake),
  Caan->Eddie Murphy (Long Island), Saget->Hall & Oates (Temple).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ajJRqKa1DUy4iKHJKPEi3
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-08-12-cinderella-contacts.xlsx
+++ b/cinderella/Outputs/2026-08-12-cinderella-contacts.xlsx
@@ -9815,7 +9815,7 @@
       <c r="D7" s="3" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Bob Newhart</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Tommy Heinsohn</t>
+          <t>Billy Collins</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -10351,7 +10351,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Bob Saget</t>
+          <t>Hall &amp; Oates</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -10403,7 +10403,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Roy Orbison</t>
+          <t>Erykah Badu</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -10576,11 +10576,7 @@
           <t>Charlie Day</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>Jay Leno</t>
-        </is>
-      </c>
+      <c r="D27" s="3" t="inlineStr"/>
       <c r="E27" s="3" t="inlineStr">
         <is>
           <t>Viola Davis</t>
@@ -10598,7 +10594,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Leno≠URI (verify)</t>
+          <t>Leno removed — no RI tie (Andover MA / LA)</t>
         </is>
       </c>
     </row>
@@ -10626,12 +10622,12 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
+          <t>Marcus Camby</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
           <t>Richard Gere</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>Jack Welch</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -11564,7 +11560,7 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Arnold Palmer</t>
+          <t>Webb Simpson</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -11640,7 +11636,7 @@
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>James Caan</t>
+          <t>Eddie Murphy</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
@@ -11759,7 +11755,7 @@
       <c r="D61" s="3" t="inlineStr"/>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Bill Walton</t>
+          <t>Mario Lopez</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Restore Jay Leno to Rhode Island — verified Newport resident (Seafair)
Correction: Leno owns the oceanfront Seafair mansion in Newport, RI
(purchased 2017). The prior 'no RI tie' removal was wrong; restored as
Rhode Island co-lead with the correct note.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ajJRqKa1DUy4iKHJKPEi3
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-08-12-cinderella-contacts.xlsx
+++ b/cinderella/Outputs/2026-08-12-cinderella-contacts.xlsx
@@ -10576,7 +10576,11 @@
           <t>Charlie Day</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Jay Leno</t>
+        </is>
+      </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
           <t>Viola Davis</t>
@@ -10594,7 +10598,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Leno removed — no RI tie (Andover MA / LA)</t>
+          <t>Leno = Newport RI resident (Seafair mansion, Ocean Ave)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add iMessage/text-outreach pass: 72 contacts + core-team cells
Combed MacBook chat.db (Jan-Aug 2026), resolved handles against Contacts,
and folded in Cinderella text contacts the Gmail pass missed:
- 4 new iMessage categories (Schools/Coaches/GMs, Reps/Talent/Production,
  Capital/Investors, Advisors/Connectors) = 72 rows.
- Cells added for Sunjay, Ankur, Greg Kristof, Jesse Jacobs, Deepen Parikh,
  Ben Simon. Confirmed Joe Mihalich title = SJU GM.
DB now 315 contacts.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ajJRqKa1DUy4iKHJKPEi3
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-08-12-cinderella-contacts.xlsx
+++ b/cinderella/Outputs/2026-08-12-cinderella-contacts.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G253"/>
+  <dimension ref="A1:G329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -531,12 +531,12 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>sunjay.mathews@gmail.com</t>
+          <t>sunjay.mathews@gmail.com / cell +1 973-464-6905</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>On nearly every thread since inception</t>
+          <t>On nearly every thread (414 texts since inception)</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>ankur08@gmail.com</t>
+          <t>ankur08@gmail.com / cell +1 917-445-1215</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>greg@6sc.io</t>
+          <t>greg@6sc.io / cell +1 508-692-0121</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -955,7 +955,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Deepen (confirm surname)</t>
+          <t>Deepen Parikh</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -965,17 +965,17 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Set the Courtside call</t>
+          <t>Partner — set the Courtside call</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>deepen@courtsidevc.com</t>
+          <t>deepen@courtsidevc.com / cell +1 443-562-2282</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Courtside organizer</t>
+          <t>Courtside; also knows Jesse/Jason at SC</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>jj@cherninent.com</t>
+          <t>jj@cherninent.com / cell +1 323-243-0157</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1673,17 +1673,17 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Ben.Simon@gs.com</t>
+          <t>Ben.Simon@gs.com / cell +1 978-399-3434</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Cold outreach</t>
+          <t>Courtside term-sheet update (text)</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -9520,16 +9520,2712 @@
         </is>
       </c>
     </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>iMessage — Schools, Coaches &amp; GMs (2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="3" t="inlineStr">
+        <is>
+          <t>Joe Mihalich</t>
+        </is>
+      </c>
+      <c r="B255" s="3" t="inlineStr">
+        <is>
+          <t>Saint Joseph's</t>
+        </is>
+      </c>
+      <c r="C255" s="3" t="inlineStr">
+        <is>
+          <t>General Manager</t>
+        </is>
+      </c>
+      <c r="D255" s="3" t="inlineStr">
+        <is>
+          <t>+1 716-807-1899 / jmihalich@sju.edu</t>
+        </is>
+      </c>
+      <c r="E255" s="3" t="inlineStr">
+        <is>
+          <t>'This is Joe Mihalich, GM at SJU'; Norman editing Hart deck Temple→SJU for him</t>
+        </is>
+      </c>
+      <c r="F255" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="G255" s="3" t="inlineStr">
+        <is>
+          <t>HOT — SJU GM, active</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="3" t="inlineStr">
+        <is>
+          <t>Chris Clunie</t>
+        </is>
+      </c>
+      <c r="B256" s="3" t="inlineStr">
+        <is>
+          <t>Davidson</t>
+        </is>
+      </c>
+      <c r="C256" s="3" t="inlineStr">
+        <is>
+          <t>Athletic Director</t>
+        </is>
+      </c>
+      <c r="D256" s="3" t="inlineStr">
+        <is>
+          <t>+1 201-328-7311</t>
+        </is>
+      </c>
+      <c r="E256" s="3" t="inlineStr">
+        <is>
+          <t>Aug touch-base ('guys are overseas')</t>
+        </is>
+      </c>
+      <c r="F256" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G256" s="3" t="inlineStr">
+        <is>
+          <t>Active — Davidson AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="3" t="inlineStr">
+        <is>
+          <t>Nathan Davis</t>
+        </is>
+      </c>
+      <c r="B257" s="3" t="inlineStr">
+        <is>
+          <t>New Hampshire</t>
+        </is>
+      </c>
+      <c r="C257" s="3" t="inlineStr">
+        <is>
+          <t>Head Coach</t>
+        </is>
+      </c>
+      <c r="D257" s="3" t="inlineStr">
+        <is>
+          <t>+1 570-238-2912</t>
+        </is>
+      </c>
+      <c r="E257" s="3" t="inlineStr">
+        <is>
+          <t>Sandler/UNH deck + LOI draft</t>
+        </is>
+      </c>
+      <c r="F257" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="G257" s="3" t="inlineStr">
+        <is>
+          <t>Active — UNH HC (Sandler school)</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="3" t="inlineStr">
+        <is>
+          <t>Kevin Young</t>
+        </is>
+      </c>
+      <c r="B258" s="3" t="inlineStr">
+        <is>
+          <t>BYU (ex-Sixers/87ers)</t>
+        </is>
+      </c>
+      <c r="C258" s="3" t="inlineStr">
+        <is>
+          <t>Head Coach</t>
+        </is>
+      </c>
+      <c r="D258" s="3" t="inlineStr">
+        <is>
+          <t>+1 678-754-6191</t>
+        </is>
+      </c>
+      <c r="E258" s="3" t="inlineStr">
+        <is>
+          <t>Soundboard; 'Steph &amp; Davidson' update</t>
+        </is>
+      </c>
+      <c r="F258" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="G258" s="3" t="inlineStr">
+        <is>
+          <t>Warm — coach ally</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="3" t="inlineStr">
+        <is>
+          <t>Dan Lobacz</t>
+        </is>
+      </c>
+      <c r="B259" s="3" t="inlineStr">
+        <is>
+          <t>Temple</t>
+        </is>
+      </c>
+      <c r="C259" s="3" t="inlineStr">
+        <is>
+          <t>Staff / NIL</t>
+        </is>
+      </c>
+      <c r="D259" s="3" t="inlineStr">
+        <is>
+          <t>+1 607-237-5849</t>
+        </is>
+      </c>
+      <c r="E259" s="3" t="inlineStr">
+        <is>
+          <t>Sent LOI draft; chasing confirm</t>
+        </is>
+      </c>
+      <c r="F259" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="G259" s="3" t="inlineStr">
+        <is>
+          <t>Active — Temple LOI</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="3" t="inlineStr">
+        <is>
+          <t>Seth Needle</t>
+        </is>
+      </c>
+      <c r="B260" s="3" t="inlineStr">
+        <is>
+          <t>(SJU/Temple connect)</t>
+        </is>
+      </c>
+      <c r="C260" s="3" t="inlineStr">
+        <is>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="D260" s="3" t="inlineStr">
+        <is>
+          <t>+1 610-761-0283</t>
+        </is>
+      </c>
+      <c r="E260" s="3" t="inlineStr">
+        <is>
+          <t>'connect me w/ Andy / Coach Fisher'; call w/ St Joe's</t>
+        </is>
+      </c>
+      <c r="F260" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G260" s="3" t="inlineStr">
+        <is>
+          <t>Active — SJU connect</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="3" t="inlineStr">
+        <is>
+          <t>Dwyane Jones</t>
+        </is>
+      </c>
+      <c r="B261" s="3" t="inlineStr">
+        <is>
+          <t>(ex-NBA / Philly)</t>
+        </is>
+      </c>
+      <c r="C261" s="3" t="inlineStr">
+        <is>
+          <t>St. Joe's connect</t>
+        </is>
+      </c>
+      <c r="D261" s="3" t="inlineStr">
+        <is>
+          <t>+1 610-636-4360</t>
+        </is>
+      </c>
+      <c r="E261" s="3" t="inlineStr">
+        <is>
+          <t>'87ers, Kevin Young staff'; SJU-related</t>
+        </is>
+      </c>
+      <c r="F261" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G261" s="3" t="inlineStr">
+        <is>
+          <t>Warm — SJU connect</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="3" t="inlineStr">
+        <is>
+          <t>Dave Paulsen</t>
+        </is>
+      </c>
+      <c r="B262" s="3" t="inlineStr">
+        <is>
+          <t>(college HC)</t>
+        </is>
+      </c>
+      <c r="C262" s="3" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="D262" s="3" t="inlineStr">
+        <is>
+          <t>+1 570-428-5520</t>
+        </is>
+      </c>
+      <c r="E262" s="3" t="inlineStr">
+        <is>
+          <t>Sent deck; 'trustees here this weekend'</t>
+        </is>
+      </c>
+      <c r="F262" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="G262" s="3" t="inlineStr">
+        <is>
+          <t>Warm — coach</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="3" t="inlineStr">
+        <is>
+          <t>Hernando Planells</t>
+        </is>
+      </c>
+      <c r="B263" s="3" t="inlineStr">
+        <is>
+          <t>(college coach)</t>
+        </is>
+      </c>
+      <c r="C263" s="3" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="D263" s="3" t="inlineStr">
+        <is>
+          <t>+1 919-972-9207</t>
+        </is>
+      </c>
+      <c r="E263" s="3" t="inlineStr">
+        <is>
+          <t>Golf-tourney reconnect</t>
+        </is>
+      </c>
+      <c r="F263" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="G263" s="3" t="inlineStr">
+        <is>
+          <t>Warm — coach</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="3" t="inlineStr">
+        <is>
+          <t>Ted Hotaling</t>
+        </is>
+      </c>
+      <c r="B264" s="3" t="inlineStr">
+        <is>
+          <t>(college coach)</t>
+        </is>
+      </c>
+      <c r="C264" s="3" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="D264" s="3" t="inlineStr">
+        <is>
+          <t>+1 203-444-7544</t>
+        </is>
+      </c>
+      <c r="E264" s="3" t="inlineStr">
+        <is>
+          <t>'congrats on D1 transition' cold update</t>
+        </is>
+      </c>
+      <c r="F264" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G264" s="3" t="inlineStr">
+        <is>
+          <t>Cold — coach</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="3" t="inlineStr">
+        <is>
+          <t>Doug Stewart</t>
+        </is>
+      </c>
+      <c r="B265" s="3" t="inlineStr">
+        <is>
+          <t>(college coach)</t>
+        </is>
+      </c>
+      <c r="C265" s="3" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="D265" s="3" t="inlineStr">
+        <is>
+          <t>+1 856-261-3313</t>
+        </is>
+      </c>
+      <c r="E265" s="3" t="inlineStr">
+        <is>
+          <t>'coach! pick your brain' early concept</t>
+        </is>
+      </c>
+      <c r="F265" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="G265" s="3" t="inlineStr">
+        <is>
+          <t>Cold — coach</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="3" t="inlineStr">
+        <is>
+          <t>Nolan Smith</t>
+        </is>
+      </c>
+      <c r="B266" s="3" t="inlineStr">
+        <is>
+          <t>(Duke/Louisville asst)</t>
+        </is>
+      </c>
+      <c r="C266" s="3" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="D266" s="3" t="inlineStr">
+        <is>
+          <t>+1 202-805-6947</t>
+        </is>
+      </c>
+      <c r="E266" s="3" t="inlineStr">
+        <is>
+          <t>'assistant from your Delaware 87ers days'</t>
+        </is>
+      </c>
+      <c r="F266" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G266" s="3" t="inlineStr">
+        <is>
+          <t>Cold — coach</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="3" t="inlineStr">
+        <is>
+          <t>Jim McGonigle</t>
+        </is>
+      </c>
+      <c r="B267" s="3" t="inlineStr">
+        <is>
+          <t>(Holy Cross connect)</t>
+        </is>
+      </c>
+      <c r="C267" s="3" t="inlineStr">
+        <is>
+          <t>HC connect</t>
+        </is>
+      </c>
+      <c r="D267" s="3" t="inlineStr">
+        <is>
+          <t>+1 508-287-7059</t>
+        </is>
+      </c>
+      <c r="E267" s="3" t="inlineStr">
+        <is>
+          <t>'HC doesn't want to be an NIL school'</t>
+        </is>
+      </c>
+      <c r="F267" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-04</t>
+        </is>
+      </c>
+      <c r="G267" s="3" t="inlineStr">
+        <is>
+          <t>Cold — HC angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>iMessage — Celebrity Reps, Talent &amp; Production (2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="3" t="inlineStr">
+        <is>
+          <t>'Boss' Everline</t>
+        </is>
+      </c>
+      <c r="B269" s="3" t="inlineStr">
+        <is>
+          <t>Hartbeat Ventures (Kevin Hart)</t>
+        </is>
+      </c>
+      <c r="C269" s="3" t="inlineStr">
+        <is>
+          <t>Exec</t>
+        </is>
+      </c>
+      <c r="D269" s="3" t="inlineStr">
+        <is>
+          <t>+1 405-423-7699 (saved 'Aaron Paul')</t>
+        </is>
+      </c>
+      <c r="E269" s="3" t="inlineStr">
+        <is>
+          <t>'you got Boss Everline from Hartbeat here, let's chat'</t>
+        </is>
+      </c>
+      <c r="F269" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="G269" s="3" t="inlineStr">
+        <is>
+          <t>HOT — Hart/Hartbeat</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="3" t="inlineStr">
+        <is>
+          <t>Justin Huchel</t>
+        </is>
+      </c>
+      <c r="B270" s="3" t="inlineStr">
+        <is>
+          <t>(Timberlake path)</t>
+        </is>
+      </c>
+      <c r="C270" s="3" t="inlineStr">
+        <is>
+          <t>Talent connector</t>
+        </is>
+      </c>
+      <c r="D270" s="3" t="inlineStr">
+        <is>
+          <t>+1 310-617-4824</t>
+        </is>
+      </c>
+      <c r="E270" s="3" t="inlineStr">
+        <is>
+          <t>Gauging JT interest as lead; wants JT-specific deck</t>
+        </is>
+      </c>
+      <c r="F270" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="G270" s="3" t="inlineStr">
+        <is>
+          <t>Active — JT path</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="3" t="inlineStr">
+        <is>
+          <t>Mike Herren</t>
+        </is>
+      </c>
+      <c r="B271" s="3" t="inlineStr">
+        <is>
+          <t>(Timberlake path)</t>
+        </is>
+      </c>
+      <c r="C271" s="3" t="inlineStr">
+        <is>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="D271" s="3" t="inlineStr">
+        <is>
+          <t>+1 508-840-5635</t>
+        </is>
+      </c>
+      <c r="E271" s="3" t="inlineStr">
+        <is>
+          <t>'I got u Timberlake guy'</t>
+        </is>
+      </c>
+      <c r="F271" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="G271" s="3" t="inlineStr">
+        <is>
+          <t>Active — JT path</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="3" t="inlineStr">
+        <is>
+          <t>Max Rudman</t>
+        </is>
+      </c>
+      <c r="B272" s="3" t="inlineStr">
+        <is>
+          <t>(talent agent)</t>
+        </is>
+      </c>
+      <c r="C272" s="3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D272" s="3" t="inlineStr">
+        <is>
+          <t>+1 847-910-0603</t>
+        </is>
+      </c>
+      <c r="E272" s="3" t="inlineStr">
+        <is>
+          <t>'send John-specific deck'</t>
+        </is>
+      </c>
+      <c r="F272" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="G272" s="3" t="inlineStr">
+        <is>
+          <t>Warm — agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="3" t="inlineStr">
+        <is>
+          <t>Zach Chu</t>
+        </is>
+      </c>
+      <c r="B273" s="3" t="inlineStr">
+        <is>
+          <t>(deck/design collaborator)</t>
+        </is>
+      </c>
+      <c r="C273" s="3" t="inlineStr">
+        <is>
+          <t>Creative</t>
+        </is>
+      </c>
+      <c r="D273" s="3" t="inlineStr">
+        <is>
+          <t>+1 214-364-9224</t>
+        </is>
+      </c>
+      <c r="E273" s="3" t="inlineStr">
+        <is>
+          <t>Builds celeb decks (Glenn Powell); La Salle board</t>
+        </is>
+      </c>
+      <c r="F273" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="G273" s="3" t="inlineStr">
+        <is>
+          <t>Active — collaborator</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="3" t="inlineStr">
+        <is>
+          <t>David Sherman</t>
+        </is>
+      </c>
+      <c r="B274" s="3" t="inlineStr">
+        <is>
+          <t>WME</t>
+        </is>
+      </c>
+      <c r="C274" s="3" t="inlineStr">
+        <is>
+          <t>Agent (non-scripted)</t>
+        </is>
+      </c>
+      <c r="D274" s="3" t="inlineStr">
+        <is>
+          <t>+1 323-445-4925</t>
+        </is>
+      </c>
+      <c r="E274" s="3" t="inlineStr">
+        <is>
+          <t>Steph-specific deck</t>
+        </is>
+      </c>
+      <c r="F274" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="G274" s="3" t="inlineStr">
+        <is>
+          <t>Warm — WME (also in vault)</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="3" t="inlineStr">
+        <is>
+          <t>Bill Straus</t>
+        </is>
+      </c>
+      <c r="B275" s="3" t="inlineStr">
+        <is>
+          <t>(music / production)</t>
+        </is>
+      </c>
+      <c r="C275" s="3" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="D275" s="3" t="inlineStr">
+        <is>
+          <t>+1 310-962-8103</t>
+        </is>
+      </c>
+      <c r="E275" s="3" t="inlineStr">
+        <is>
+          <t>Production-deck; 'vinyl, NWA'</t>
+        </is>
+      </c>
+      <c r="F275" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="G275" s="3" t="inlineStr">
+        <is>
+          <t>Active — production</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="3" t="inlineStr">
+        <is>
+          <t>Alexandre Rockwell</t>
+        </is>
+      </c>
+      <c r="B276" s="3" t="inlineStr">
+        <is>
+          <t>(film director)</t>
+        </is>
+      </c>
+      <c r="C276" s="3" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="D276" s="3" t="inlineStr">
+        <is>
+          <t>+1 310-415-2305</t>
+        </is>
+      </c>
+      <c r="E276" s="3" t="inlineStr">
+        <is>
+          <t>'learning the production world'; LOI update</t>
+        </is>
+      </c>
+      <c r="F276" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="G276" s="3" t="inlineStr">
+        <is>
+          <t>Active — production</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="3" t="inlineStr">
+        <is>
+          <t>Lilly Burns</t>
+        </is>
+      </c>
+      <c r="B277" s="3" t="inlineStr">
+        <is>
+          <t>Jax Media</t>
+        </is>
+      </c>
+      <c r="C277" s="3" t="inlineStr">
+        <is>
+          <t>TV producer</t>
+        </is>
+      </c>
+      <c r="D277" s="3" t="inlineStr">
+        <is>
+          <t>+1 917-587-7523</t>
+        </is>
+      </c>
+      <c r="E277" s="3" t="inlineStr">
+        <is>
+          <t>Loomis classmate; producer</t>
+        </is>
+      </c>
+      <c r="F277" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="G277" s="3" t="inlineStr">
+        <is>
+          <t>Warm — producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="3" t="inlineStr">
+        <is>
+          <t>Scott Manson</t>
+        </is>
+      </c>
+      <c r="B278" s="3" t="inlineStr">
+        <is>
+          <t>SpringHill / UNINTERRUPTED (LeBron)</t>
+        </is>
+      </c>
+      <c r="C278" s="3" t="inlineStr">
+        <is>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="D278" s="3" t="inlineStr">
+        <is>
+          <t>+1 310-270-6094</t>
+        </is>
+      </c>
+      <c r="E278" s="3" t="inlineStr">
+        <is>
+          <t>SOFI / NIL marketing</t>
+        </is>
+      </c>
+      <c r="F278" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="G278" s="3" t="inlineStr">
+        <is>
+          <t>Warm — LeBron-adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="3" t="inlineStr">
+        <is>
+          <t>TJ McConnell</t>
+        </is>
+      </c>
+      <c r="B279" s="3" t="inlineStr">
+        <is>
+          <t>Indiana Pacers (NBA)</t>
+        </is>
+      </c>
+      <c r="C279" s="3" t="inlineStr">
+        <is>
+          <t>Talent/connector</t>
+        </is>
+      </c>
+      <c r="D279" s="3" t="inlineStr">
+        <is>
+          <t>+1 412-980-2620</t>
+        </is>
+      </c>
+      <c r="E279" s="3" t="inlineStr">
+        <is>
+          <t>'meeting Hart's team re Temple/St Joe's'</t>
+        </is>
+      </c>
+      <c r="F279" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="G279" s="3" t="inlineStr">
+        <is>
+          <t>Warm — NBA connect</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="3" t="inlineStr">
+        <is>
+          <t>Chris Herren</t>
+        </is>
+      </c>
+      <c r="B280" s="3" t="inlineStr">
+        <is>
+          <t>(ex-NBA / speaker)</t>
+        </is>
+      </c>
+      <c r="C280" s="3" t="inlineStr">
+        <is>
+          <t>Talent/connector</t>
+        </is>
+      </c>
+      <c r="D280" s="3" t="inlineStr">
+        <is>
+          <t>+1 401-626-2445</t>
+        </is>
+      </c>
+      <c r="E280" s="3" t="inlineStr">
+        <is>
+          <t>Intro via Mike; NIL project</t>
+        </is>
+      </c>
+      <c r="F280" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="G280" s="3" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="3" t="inlineStr">
+        <is>
+          <t>Josh Altman</t>
+        </is>
+      </c>
+      <c r="B281" s="3" t="inlineStr">
+        <is>
+          <t>(Million Dollar Listing)</t>
+        </is>
+      </c>
+      <c r="C281" s="3" t="inlineStr">
+        <is>
+          <t>Talent/connector</t>
+        </is>
+      </c>
+      <c r="D281" s="3" t="inlineStr">
+        <is>
+          <t>+1 323-610-0231</t>
+        </is>
+      </c>
+      <c r="E281" s="3" t="inlineStr">
+        <is>
+          <t>'need a celeb' pitch</t>
+        </is>
+      </c>
+      <c r="F281" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="G281" s="3" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="3" t="inlineStr">
+        <is>
+          <t>Ken Jeong</t>
+        </is>
+      </c>
+      <c r="B282" s="3" t="inlineStr">
+        <is>
+          <t>(actor)</t>
+        </is>
+      </c>
+      <c r="C282" s="3" t="inlineStr">
+        <is>
+          <t>Talent</t>
+        </is>
+      </c>
+      <c r="D282" s="3" t="inlineStr">
+        <is>
+          <t>+1 310-779-8260</t>
+        </is>
+      </c>
+      <c r="E282" s="3" t="inlineStr">
+        <is>
+          <t>Steph/Davidson update</t>
+        </is>
+      </c>
+      <c r="F282" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="G282" s="3" t="inlineStr">
+        <is>
+          <t>Cold — talent</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="3" t="inlineStr">
+        <is>
+          <t>Jordan Fliegel</t>
+        </is>
+      </c>
+      <c r="B283" s="3" t="inlineStr">
+        <is>
+          <t>(CoachUp founder / VC)</t>
+        </is>
+      </c>
+      <c r="C283" s="3" t="inlineStr">
+        <is>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="D283" s="3" t="inlineStr">
+        <is>
+          <t>+1 617-943-8750</t>
+        </is>
+      </c>
+      <c r="E283" s="3" t="inlineStr">
+        <is>
+          <t>'congrats on Miami move, new business'</t>
+        </is>
+      </c>
+      <c r="F283" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="G283" s="3" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="3" t="inlineStr">
+        <is>
+          <t>Tim Grover</t>
+        </is>
+      </c>
+      <c r="B284" s="3" t="inlineStr">
+        <is>
+          <t>(trainer — MJ/Kobe)</t>
+        </is>
+      </c>
+      <c r="C284" s="3" t="inlineStr">
+        <is>
+          <t>Trainer/rep</t>
+        </is>
+      </c>
+      <c r="D284" s="3" t="inlineStr">
+        <is>
+          <t>+1 312-823-2320</t>
+        </is>
+      </c>
+      <c r="E284" s="3" t="inlineStr">
+        <is>
+          <t>Cold concept pitch</t>
+        </is>
+      </c>
+      <c r="F284" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="G284" s="3" t="inlineStr">
+        <is>
+          <t>Cold — trainer</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="3" t="inlineStr">
+        <is>
+          <t>Rod Baker</t>
+        </is>
+      </c>
+      <c r="B285" s="3" t="inlineStr">
+        <is>
+          <t>(MSA-adjacent)</t>
+        </is>
+      </c>
+      <c r="C285" s="3" t="inlineStr">
+        <is>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="D285" s="3" t="inlineStr">
+        <is>
+          <t>+1 585-451-3235</t>
+        </is>
+      </c>
+      <c r="E285" s="3" t="inlineStr">
+        <is>
+          <t>'MSA floated LeBron/Akron'</t>
+        </is>
+      </c>
+      <c r="F285" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="G285" s="3" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>iMessage — Capital &amp; Investors (2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="3" t="inlineStr">
+        <is>
+          <t>Josh Bennett</t>
+        </is>
+      </c>
+      <c r="B287" s="3" t="inlineStr">
+        <is>
+          <t>(investor, NH)</t>
+        </is>
+      </c>
+      <c r="C287" s="3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="D287" s="3" t="inlineStr">
+        <is>
+          <t>+1 603-387-2068</t>
+        </is>
+      </c>
+      <c r="E287" s="3" t="inlineStr">
+        <is>
+          <t>'deck received, keep chatting'</t>
+        </is>
+      </c>
+      <c r="F287" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="G287" s="3" t="inlineStr">
+        <is>
+          <t>Active — investor</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="3" t="inlineStr">
+        <is>
+          <t>Alan Chang</t>
+        </is>
+      </c>
+      <c r="B288" s="3" t="inlineStr">
+        <is>
+          <t>(sports-biz investor)</t>
+        </is>
+      </c>
+      <c r="C288" s="3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="D288" s="3" t="inlineStr">
+        <is>
+          <t>+1 702-292-5700</t>
+        </is>
+      </c>
+      <c r="E288" s="3" t="inlineStr">
+        <is>
+          <t>Deck Qs on celeb comp</t>
+        </is>
+      </c>
+      <c r="F288" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="G288" s="3" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="3" t="inlineStr">
+        <is>
+          <t>Noah Yates</t>
+        </is>
+      </c>
+      <c r="B289" s="3" t="inlineStr">
+        <is>
+          <t>Y Investments</t>
+        </is>
+      </c>
+      <c r="C289" s="3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="D289" s="3" t="inlineStr">
+        <is>
+          <t>+1 732-608-3499</t>
+        </is>
+      </c>
+      <c r="E289" s="3" t="inlineStr">
+        <is>
+          <t>'no bandwidth for parentco right now'</t>
+        </is>
+      </c>
+      <c r="F289" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="G289" s="3" t="inlineStr">
+        <is>
+          <t>Passed — revisit</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="3" t="inlineStr">
+        <is>
+          <t>Jay Jackson</t>
+        </is>
+      </c>
+      <c r="B290" s="3" t="inlineStr">
+        <is>
+          <t>(principal / advisor)</t>
+        </is>
+      </c>
+      <c r="C290" s="3" t="inlineStr">
+        <is>
+          <t>Advisor</t>
+        </is>
+      </c>
+      <c r="D290" s="3" t="inlineStr">
+        <is>
+          <t>+1 310-503-0419</t>
+        </is>
+      </c>
+      <c r="E290" s="3" t="inlineStr">
+        <is>
+          <t>Formal comms; input on names</t>
+        </is>
+      </c>
+      <c r="F290" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G290" s="3" t="inlineStr">
+        <is>
+          <t>Active — advisor</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="3" t="inlineStr">
+        <is>
+          <t>Tyler Glass</t>
+        </is>
+      </c>
+      <c r="B291" s="3" t="inlineStr">
+        <is>
+          <t>(investor/advisor)</t>
+        </is>
+      </c>
+      <c r="C291" s="3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="D291" s="3" t="inlineStr">
+        <is>
+          <t>+1 201-563-1919</t>
+        </is>
+      </c>
+      <c r="E291" s="3" t="inlineStr">
+        <is>
+          <t>'this is fantastic — how I envisioned it'</t>
+        </is>
+      </c>
+      <c r="F291" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="G291" s="3" t="inlineStr">
+        <is>
+          <t>Warm — enthusiastic</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="3" t="inlineStr">
+        <is>
+          <t>Jameson Davis</t>
+        </is>
+      </c>
+      <c r="B292" s="3" t="inlineStr">
+        <is>
+          <t>DraftKings (VIP)</t>
+        </is>
+      </c>
+      <c r="C292" s="3" t="inlineStr">
+        <is>
+          <t>Connector/investor</t>
+        </is>
+      </c>
+      <c r="D292" s="3" t="inlineStr">
+        <is>
+          <t>+1 617-631-2530</t>
+        </is>
+      </c>
+      <c r="E292" s="3" t="inlineStr">
+        <is>
+          <t>Early concept</t>
+        </is>
+      </c>
+      <c r="F292" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="G292" s="3" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="3" t="inlineStr">
+        <is>
+          <t>Esteban Arguello</t>
+        </is>
+      </c>
+      <c r="B293" s="3" t="inlineStr">
+        <is>
+          <t>(investor)</t>
+        </is>
+      </c>
+      <c r="C293" s="3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="D293" s="3" t="inlineStr">
+        <is>
+          <t>+1 661-993-8226</t>
+        </is>
+      </c>
+      <c r="E293" s="3" t="inlineStr">
+        <is>
+          <t>Deck + numbers</t>
+        </is>
+      </c>
+      <c r="F293" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G293" s="3" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="3" t="inlineStr">
+        <is>
+          <t>Michael Siegel</t>
+        </is>
+      </c>
+      <c r="B294" s="3" t="inlineStr">
+        <is>
+          <t>(investor)</t>
+        </is>
+      </c>
+      <c r="C294" s="3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="D294" s="3" t="inlineStr">
+        <is>
+          <t>+1 610-517-3836</t>
+        </is>
+      </c>
+      <c r="E294" s="3" t="inlineStr">
+        <is>
+          <t>Coaches-NIL venture</t>
+        </is>
+      </c>
+      <c r="F294" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="G294" s="3" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="3" t="inlineStr">
+        <is>
+          <t>Gibson Johnson</t>
+        </is>
+      </c>
+      <c r="B295" s="3" t="inlineStr">
+        <is>
+          <t>(investor)</t>
+        </is>
+      </c>
+      <c r="C295" s="3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="D295" s="3" t="inlineStr">
+        <is>
+          <t>+1 385-209-4481</t>
+        </is>
+      </c>
+      <c r="E295" s="3" t="inlineStr">
+        <is>
+          <t>/dj deck</t>
+        </is>
+      </c>
+      <c r="F295" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="G295" s="3" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="3" t="inlineStr">
+        <is>
+          <t>Jonathan Chang</t>
+        </is>
+      </c>
+      <c r="B296" s="3" t="inlineStr">
+        <is>
+          <t>(investor, Seattle)</t>
+        </is>
+      </c>
+      <c r="C296" s="3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="D296" s="3" t="inlineStr">
+        <is>
+          <t>+1 425-894-5051</t>
+        </is>
+      </c>
+      <c r="E296" s="3" t="inlineStr">
+        <is>
+          <t>Steph/Davidson news; term-sheet interest</t>
+        </is>
+      </c>
+      <c r="F296" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="G296" s="3" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="3" t="inlineStr">
+        <is>
+          <t>Kevin Hussey</t>
+        </is>
+      </c>
+      <c r="B297" s="3" t="inlineStr">
+        <is>
+          <t>(investor/connector)</t>
+        </is>
+      </c>
+      <c r="C297" s="3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="D297" s="3" t="inlineStr">
+        <is>
+          <t>+1 310-499-8239</t>
+        </is>
+      </c>
+      <c r="E297" s="3" t="inlineStr">
+        <is>
+          <t>RedBird NYC meeting</t>
+        </is>
+      </c>
+      <c r="F297" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="G297" s="3" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="3" t="inlineStr">
+        <is>
+          <t>Kevin Volchok</t>
+        </is>
+      </c>
+      <c r="B298" s="3" t="inlineStr">
+        <is>
+          <t>(investor/advisor)</t>
+        </is>
+      </c>
+      <c r="C298" s="3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="D298" s="3" t="inlineStr">
+        <is>
+          <t>+1 310-508-5000</t>
+        </is>
+      </c>
+      <c r="E298" s="3" t="inlineStr">
+        <is>
+          <t>Portal timing</t>
+        </is>
+      </c>
+      <c r="F298" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="G298" s="3" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="3" t="inlineStr">
+        <is>
+          <t>Brendan Greeley</t>
+        </is>
+      </c>
+      <c r="B299" s="3" t="inlineStr">
+        <is>
+          <t>(investor/advisor)</t>
+        </is>
+      </c>
+      <c r="C299" s="3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="D299" s="3" t="inlineStr">
+        <is>
+          <t>+1 312-330-5316</t>
+        </is>
+      </c>
+      <c r="E299" s="3" t="inlineStr">
+        <is>
+          <t>Docu-series structure</t>
+        </is>
+      </c>
+      <c r="F299" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="G299" s="3" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="3" t="inlineStr">
+        <is>
+          <t>Gregory Bush</t>
+        </is>
+      </c>
+      <c r="B300" s="3" t="inlineStr">
+        <is>
+          <t>(investor)</t>
+        </is>
+      </c>
+      <c r="C300" s="3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="D300" s="3" t="inlineStr">
+        <is>
+          <t>+1 631-495-4763</t>
+        </is>
+      </c>
+      <c r="E300" s="3" t="inlineStr">
+        <is>
+          <t>'raised $12M' pitch</t>
+        </is>
+      </c>
+      <c r="F300" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="G300" s="3" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="3" t="inlineStr">
+        <is>
+          <t>Chad Hutchinson</t>
+        </is>
+      </c>
+      <c r="B301" s="3" t="inlineStr">
+        <is>
+          <t>(finance / ex-athlete)</t>
+        </is>
+      </c>
+      <c r="C301" s="3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="D301" s="3" t="inlineStr">
+        <is>
+          <t>+1 214-957-7861</t>
+        </is>
+      </c>
+      <c r="E301" s="3" t="inlineStr">
+        <is>
+          <t>Cold VC update</t>
+        </is>
+      </c>
+      <c r="F301" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="G301" s="3" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="3" t="inlineStr">
+        <is>
+          <t>Mike Wenzell</t>
+        </is>
+      </c>
+      <c r="B302" s="3" t="inlineStr">
+        <is>
+          <t>(China basketball)</t>
+        </is>
+      </c>
+      <c r="C302" s="3" t="inlineStr">
+        <is>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="D302" s="3" t="inlineStr">
+        <is>
+          <t>+86 185-1454-0553</t>
+        </is>
+      </c>
+      <c r="E302" s="3" t="inlineStr">
+        <is>
+          <t>'navigating the system over there'</t>
+        </is>
+      </c>
+      <c r="F302" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="G302" s="3" t="inlineStr">
+        <is>
+          <t>Warm — China</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="2" t="inlineStr">
+        <is>
+          <t>iMessage — Advisors, Connectors &amp; Soundboards (2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="3" t="inlineStr">
+        <is>
+          <t>Nate Fritsch</t>
+        </is>
+      </c>
+      <c r="B304" s="3" t="inlineStr">
+        <is>
+          <t>(advisor)</t>
+        </is>
+      </c>
+      <c r="C304" s="3" t="inlineStr">
+        <is>
+          <t>Advisor</t>
+        </is>
+      </c>
+      <c r="D304" s="3" t="inlineStr">
+        <is>
+          <t>+1 919-475-2625</t>
+        </is>
+      </c>
+      <c r="E304" s="3" t="inlineStr">
+        <is>
+          <t>Davidson / Hun / Matt McKillop connect; deck feedback</t>
+        </is>
+      </c>
+      <c r="F304" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="G304" s="3" t="inlineStr">
+        <is>
+          <t>Active — Davidson advisor (also in DB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="3" t="inlineStr">
+        <is>
+          <t>Chris Caputo</t>
+        </is>
+      </c>
+      <c r="B305" s="3" t="inlineStr">
+        <is>
+          <t>George Washington</t>
+        </is>
+      </c>
+      <c r="C305" s="3" t="inlineStr">
+        <is>
+          <t>Head Coach</t>
+        </is>
+      </c>
+      <c r="D305" s="3" t="inlineStr">
+        <is>
+          <t>+1 786-877-2864</t>
+        </is>
+      </c>
+      <c r="E305" s="3" t="inlineStr">
+        <is>
+          <t>Woj connected; LOIs Davidson/SJU</t>
+        </is>
+      </c>
+      <c r="F305" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="G305" s="3" t="inlineStr">
+        <is>
+          <t>Active — GW HC</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="3" t="inlineStr">
+        <is>
+          <t>Erick Peyton</t>
+        </is>
+      </c>
+      <c r="B306" s="3" t="inlineStr">
+        <is>
+          <t>Unanimous Media (Curry)</t>
+        </is>
+      </c>
+      <c r="C306" s="3" t="inlineStr">
+        <is>
+          <t>Principal</t>
+        </is>
+      </c>
+      <c r="D306" s="3" t="inlineStr">
+        <is>
+          <t>+1 323-899-5748</t>
+        </is>
+      </c>
+      <c r="E306" s="3" t="inlineStr">
+        <is>
+          <t>'UM / Davidson status'</t>
+        </is>
+      </c>
+      <c r="F306" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="G306" s="3" t="inlineStr">
+        <is>
+          <t>Active — Curry/Unanimous</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="3" t="inlineStr">
+        <is>
+          <t>Adrian Williams</t>
+        </is>
+      </c>
+      <c r="B307" s="3" t="inlineStr">
+        <is>
+          <t>SC Holdings</t>
+        </is>
+      </c>
+      <c r="C307" s="3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="D307" s="3" t="inlineStr">
+        <is>
+          <t>+1 404-421-0361</t>
+        </is>
+      </c>
+      <c r="E307" s="3" t="inlineStr">
+        <is>
+          <t>Relays Erick / term sheet</t>
+        </is>
+      </c>
+      <c r="F307" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="G307" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="3" t="inlineStr">
+        <is>
+          <t>Becca (Rebecca) Gitlitz</t>
+        </is>
+      </c>
+      <c r="B308" s="3" t="inlineStr">
+        <is>
+          <t>EverWonder</t>
+        </is>
+      </c>
+      <c r="C308" s="3" t="inlineStr">
+        <is>
+          <t>Exec</t>
+        </is>
+      </c>
+      <c r="D308" s="3" t="inlineStr">
+        <is>
+          <t>+1 201-669-6884</t>
+        </is>
+      </c>
+      <c r="E308" s="3" t="inlineStr">
+        <is>
+          <t>Andrew Luck/Stanford NIL tidbit</t>
+        </is>
+      </c>
+      <c r="F308" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="G308" s="3" t="inlineStr">
+        <is>
+          <t>Active — EverWonder</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="3" t="inlineStr">
+        <is>
+          <t>Deirdre Fenton</t>
+        </is>
+      </c>
+      <c r="B309" s="3" t="inlineStr">
+        <is>
+          <t>EverWonder</t>
+        </is>
+      </c>
+      <c r="C309" s="3" t="inlineStr">
+        <is>
+          <t>Exec</t>
+        </is>
+      </c>
+      <c r="D309" s="3" t="inlineStr">
+        <is>
+          <t>+1 646-275-6540</t>
+        </is>
+      </c>
+      <c r="E309" s="3" t="inlineStr">
+        <is>
+          <t>Intro thread</t>
+        </is>
+      </c>
+      <c r="F309" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="G309" s="3" t="inlineStr">
+        <is>
+          <t>Active — EverWonder</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="3" t="inlineStr">
+        <is>
+          <t>Eric Newman</t>
+        </is>
+      </c>
+      <c r="B310" s="3" t="inlineStr">
+        <is>
+          <t>(production via Donahue)</t>
+        </is>
+      </c>
+      <c r="C310" s="3" t="inlineStr">
+        <is>
+          <t>Producer</t>
+        </is>
+      </c>
+      <c r="D310" s="3" t="inlineStr">
+        <is>
+          <t>+1 516-965-3507</t>
+        </is>
+      </c>
+      <c r="E310" s="3" t="inlineStr">
+        <is>
+          <t>Meeting set w/ Sunjay</t>
+        </is>
+      </c>
+      <c r="F310" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="G310" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="3" t="inlineStr">
+        <is>
+          <t>Jeremy Peschka</t>
+        </is>
+      </c>
+      <c r="B311" s="3" t="inlineStr">
+        <is>
+          <t>(media/connector)</t>
+        </is>
+      </c>
+      <c r="C311" s="3" t="inlineStr">
+        <is>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="D311" s="3" t="inlineStr">
+        <is>
+          <t>+1 971-285-6078</t>
+        </is>
+      </c>
+      <c r="E311" s="3" t="inlineStr">
+        <is>
+          <t>Peacock docuseries intel; Kevin O'Leary path</t>
+        </is>
+      </c>
+      <c r="F311" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="G311" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="3" t="inlineStr">
+        <is>
+          <t>Varun Sudhakar</t>
+        </is>
+      </c>
+      <c r="B312" s="3" t="inlineStr">
+        <is>
+          <t>(advisor, UK)</t>
+        </is>
+      </c>
+      <c r="C312" s="3" t="inlineStr">
+        <is>
+          <t>Advisor / model</t>
+        </is>
+      </c>
+      <c r="D312" s="3" t="inlineStr">
+        <is>
+          <t>+1 609-433-1085</t>
+        </is>
+      </c>
+      <c r="E312" s="3" t="inlineStr">
+        <is>
+          <t>Works the financial model; USC-NIL contact via Nigel</t>
+        </is>
+      </c>
+      <c r="F312" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="G312" s="3" t="inlineStr">
+        <is>
+          <t>Active — model</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="3" t="inlineStr">
+        <is>
+          <t>Alex Miska</t>
+        </is>
+      </c>
+      <c r="B313" s="3" t="inlineStr">
+        <is>
+          <t>Foley &amp; Lardner</t>
+        </is>
+      </c>
+      <c r="C313" s="3" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="D313" s="3" t="inlineStr">
+        <is>
+          <t>+1 908-500-1063</t>
+        </is>
+      </c>
+      <c r="E313" s="3" t="inlineStr">
+        <is>
+          <t>'Luke Murray congrats'; term-sheet help</t>
+        </is>
+      </c>
+      <c r="F313" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="G313" s="3" t="inlineStr">
+        <is>
+          <t>Warm — legal</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="3" t="inlineStr">
+        <is>
+          <t>Shavlik Randolph</t>
+        </is>
+      </c>
+      <c r="B314" s="3" t="inlineStr">
+        <is>
+          <t>(ex-NBA)</t>
+        </is>
+      </c>
+      <c r="C314" s="3" t="inlineStr">
+        <is>
+          <t>Advisor/connector</t>
+        </is>
+      </c>
+      <c r="D314" s="3" t="inlineStr">
+        <is>
+          <t>+1 919-539-1309</t>
+        </is>
+      </c>
+      <c r="E314" s="3" t="inlineStr">
+        <is>
+          <t>Wrexham-concept riffing</t>
+        </is>
+      </c>
+      <c r="F314" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="G314" s="3" t="inlineStr">
+        <is>
+          <t>Warm — ex-NBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="3" t="inlineStr">
+        <is>
+          <t>Kevin Owens</t>
+        </is>
+      </c>
+      <c r="B315" s="3" t="inlineStr">
+        <is>
+          <t>(NIL operator)</t>
+        </is>
+      </c>
+      <c r="C315" s="3" t="inlineStr">
+        <is>
+          <t>Peer operator</t>
+        </is>
+      </c>
+      <c r="D315" s="3" t="inlineStr">
+        <is>
+          <t>+1 973-303-1637</t>
+        </is>
+      </c>
+      <c r="E315" s="3" t="inlineStr">
+        <is>
+          <t>'raised $ for NIL play'; Hart-team meetings</t>
+        </is>
+      </c>
+      <c r="F315" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G315" s="3" t="inlineStr">
+        <is>
+          <t>Warm — peer</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="3" t="inlineStr">
+        <is>
+          <t>Tom Baudinet</t>
+        </is>
+      </c>
+      <c r="B316" s="3" t="inlineStr">
+        <is>
+          <t>(advisor)</t>
+        </is>
+      </c>
+      <c r="C316" s="3" t="inlineStr">
+        <is>
+          <t>Advisor</t>
+        </is>
+      </c>
+      <c r="D316" s="3" t="inlineStr">
+        <is>
+          <t>+1 203-695-4381</t>
+        </is>
+      </c>
+      <c r="E316" s="3" t="inlineStr">
+        <is>
+          <t>'chatting with KY... NCAA/NIL insight'</t>
+        </is>
+      </c>
+      <c r="F316" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="G316" s="3" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="3" t="inlineStr">
+        <is>
+          <t>Austin Buntz</t>
+        </is>
+      </c>
+      <c r="B317" s="3" t="inlineStr">
+        <is>
+          <t>(creative)</t>
+        </is>
+      </c>
+      <c r="C317" s="3" t="inlineStr">
+        <is>
+          <t>Creative</t>
+        </is>
+      </c>
+      <c r="D317" s="3" t="inlineStr">
+        <is>
+          <t>+1 570-579-6181</t>
+        </is>
+      </c>
+      <c r="E317" s="3" t="inlineStr">
+        <is>
+          <t>Wrote Wrexham pitch; building deck w/ Jesse</t>
+        </is>
+      </c>
+      <c r="F317" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="G317" s="3" t="inlineStr">
+        <is>
+          <t>Active — creative</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="3" t="inlineStr">
+        <is>
+          <t>Dane Diliegro</t>
+        </is>
+      </c>
+      <c r="B318" s="3" t="inlineStr">
+        <is>
+          <t>(actor/athlete)</t>
+        </is>
+      </c>
+      <c r="C318" s="3" t="inlineStr">
+        <is>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="D318" s="3" t="inlineStr">
+        <is>
+          <t>+1 781-589-0820</t>
+        </is>
+      </c>
+      <c r="E318" s="3" t="inlineStr">
+        <is>
+          <t>Concept soundboard</t>
+        </is>
+      </c>
+      <c r="F318" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="G318" s="3" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="3" t="inlineStr">
+        <is>
+          <t>Steve Ceruti</t>
+        </is>
+      </c>
+      <c r="B319" s="3" t="inlineStr">
+        <is>
+          <t>Barstool (Russillo)</t>
+        </is>
+      </c>
+      <c r="C319" s="3" t="inlineStr">
+        <is>
+          <t>Media connect</t>
+        </is>
+      </c>
+      <c r="D319" s="3" t="inlineStr">
+        <is>
+          <t>+1 860-302-2869</t>
+        </is>
+      </c>
+      <c r="E319" s="3" t="inlineStr">
+        <is>
+          <t>Barstool/Russillo; Affleck-agent feedback</t>
+        </is>
+      </c>
+      <c r="F319" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="G319" s="3" t="inlineStr">
+        <is>
+          <t>Warm — media</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="3" t="inlineStr">
+        <is>
+          <t>Mike Sotsky</t>
+        </is>
+      </c>
+      <c r="B320" s="3" t="inlineStr">
+        <is>
+          <t>Harvard Basketball</t>
+        </is>
+      </c>
+      <c r="C320" s="3" t="inlineStr">
+        <is>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="D320" s="3" t="inlineStr">
+        <is>
+          <t>+1 201-956-0883</t>
+        </is>
+      </c>
+      <c r="E320" s="3" t="inlineStr">
+        <is>
+          <t>'showed TA the deck'</t>
+        </is>
+      </c>
+      <c r="F320" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="G320" s="3" t="inlineStr">
+        <is>
+          <t>Warm — Harvard</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="3" t="inlineStr">
+        <is>
+          <t>Matt Janning</t>
+        </is>
+      </c>
+      <c r="B321" s="3" t="inlineStr">
+        <is>
+          <t>(ex-pro player)</t>
+        </is>
+      </c>
+      <c r="C321" s="3" t="inlineStr">
+        <is>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="D321" s="3" t="inlineStr">
+        <is>
+          <t>+1 612-867-8797</t>
+        </is>
+      </c>
+      <c r="E321" s="3" t="inlineStr">
+        <is>
+          <t>Wahlberg proposal</t>
+        </is>
+      </c>
+      <c r="F321" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="G321" s="3" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="3" t="inlineStr">
+        <is>
+          <t>Conor Stevens</t>
+        </is>
+      </c>
+      <c r="B322" s="3" t="inlineStr">
+        <is>
+          <t>(Stevens family)</t>
+        </is>
+      </c>
+      <c r="C322" s="3" t="inlineStr">
+        <is>
+          <t>Personal ally</t>
+        </is>
+      </c>
+      <c r="D322" s="3" t="inlineStr">
+        <is>
+          <t>+1 617-610-1327</t>
+        </is>
+      </c>
+      <c r="E322" s="3" t="inlineStr">
+        <is>
+          <t>Davidson/Steph update</t>
+        </is>
+      </c>
+      <c r="F322" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="G322" s="3" t="inlineStr">
+        <is>
+          <t>Ally</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="3" t="inlineStr">
+        <is>
+          <t>Ryan Cain</t>
+        </is>
+      </c>
+      <c r="B323" s="3" t="inlineStr">
+        <is>
+          <t>(coach/friend)</t>
+        </is>
+      </c>
+      <c r="C323" s="3" t="inlineStr">
+        <is>
+          <t>Soundboard</t>
+        </is>
+      </c>
+      <c r="D323" s="3" t="inlineStr">
+        <is>
+          <t>+1 508-873-5005</t>
+        </is>
+      </c>
+      <c r="E323" s="3" t="inlineStr">
+        <is>
+          <t>School-openness question</t>
+        </is>
+      </c>
+      <c r="F323" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="G323" s="3" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="3" t="inlineStr">
+        <is>
+          <t>Joey Flannery</t>
+        </is>
+      </c>
+      <c r="B324" s="3" t="inlineStr">
+        <is>
+          <t>(peer)</t>
+        </is>
+      </c>
+      <c r="C324" s="3" t="inlineStr">
+        <is>
+          <t>Soundboard</t>
+        </is>
+      </c>
+      <c r="D324" s="3" t="inlineStr">
+        <is>
+          <t>+1 978-303-7677</t>
+        </is>
+      </c>
+      <c r="E324" s="3" t="inlineStr">
+        <is>
+          <t>Pitch narrative</t>
+        </is>
+      </c>
+      <c r="F324" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="G324" s="3" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="3" t="inlineStr">
+        <is>
+          <t>Brendan Lang</t>
+        </is>
+      </c>
+      <c r="B325" s="3" t="inlineStr">
+        <is>
+          <t>(advisor)</t>
+        </is>
+      </c>
+      <c r="C325" s="3" t="inlineStr">
+        <is>
+          <t>Advisor</t>
+        </is>
+      </c>
+      <c r="D325" s="3" t="inlineStr">
+        <is>
+          <t>+1 774-263-2705</t>
+        </is>
+      </c>
+      <c r="E325" s="3" t="inlineStr">
+        <is>
+          <t>BYU collectives insight</t>
+        </is>
+      </c>
+      <c r="F325" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="G325" s="3" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="3" t="inlineStr">
+        <is>
+          <t>Mark Palmieri</t>
+        </is>
+      </c>
+      <c r="B326" s="3" t="inlineStr">
+        <is>
+          <t>(advisor)</t>
+        </is>
+      </c>
+      <c r="C326" s="3" t="inlineStr">
+        <is>
+          <t>Advisor</t>
+        </is>
+      </c>
+      <c r="D326" s="3" t="inlineStr">
+        <is>
+          <t>+1 203-641-4518</t>
+        </is>
+      </c>
+      <c r="E326" s="3" t="inlineStr">
+        <is>
+          <t>Ivy/NIL note</t>
+        </is>
+      </c>
+      <c r="F326" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="G326" s="3" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="3" t="inlineStr">
+        <is>
+          <t>Matt Blue</t>
+        </is>
+      </c>
+      <c r="B327" s="3" t="inlineStr">
+        <is>
+          <t>(connector)</t>
+        </is>
+      </c>
+      <c r="C327" s="3" t="inlineStr">
+        <is>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="D327" s="3" t="inlineStr">
+        <is>
+          <t>+1 508-254-4752</t>
+        </is>
+      </c>
+      <c r="E327" s="3" t="inlineStr">
+        <is>
+          <t>Celeb sourcing</t>
+        </is>
+      </c>
+      <c r="F327" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G327" s="3" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="3" t="inlineStr">
+        <is>
+          <t>Arthur Lynch</t>
+        </is>
+      </c>
+      <c r="B328" s="3" t="inlineStr">
+        <is>
+          <t>(ex-NFL)</t>
+        </is>
+      </c>
+      <c r="C328" s="3" t="inlineStr">
+        <is>
+          <t>Soundboard</t>
+        </is>
+      </c>
+      <c r="D328" s="3" t="inlineStr">
+        <is>
+          <t>+1 508-369-0782</t>
+        </is>
+      </c>
+      <c r="E328" s="3" t="inlineStr">
+        <is>
+          <t>Deck review</t>
+        </is>
+      </c>
+      <c r="F328" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="G328" s="3" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="3" t="inlineStr">
+        <is>
+          <t>Cliff Furtado</t>
+        </is>
+      </c>
+      <c r="B329" s="3" t="inlineStr">
+        <is>
+          <t>(friend)</t>
+        </is>
+      </c>
+      <c r="C329" s="3" t="inlineStr">
+        <is>
+          <t>Legal referral</t>
+        </is>
+      </c>
+      <c r="D329" s="3" t="inlineStr">
+        <is>
+          <t>+1 508-491-7250</t>
+        </is>
+      </c>
+      <c r="E329" s="3" t="inlineStr">
+        <is>
+          <t>Lawyer refs for term sheet</t>
+        </is>
+      </c>
+      <c r="F329" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="G329" s="3" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
-  <mergeCells count="9">
+  <mergeCells count="13">
     <mergeCell ref="A123:G123"/>
     <mergeCell ref="A141:G141"/>
+    <mergeCell ref="A254:G254"/>
+    <mergeCell ref="A286:G286"/>
     <mergeCell ref="A97:G97"/>
+    <mergeCell ref="A303:G303"/>
     <mergeCell ref="A79:G79"/>
     <mergeCell ref="A55:G55"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A183:G183"/>
+    <mergeCell ref="A268:G268"/>
     <mergeCell ref="A10:G10"/>
     <mergeCell ref="A133:G133"/>
   </mergeCells>

</xml_diff>